<commit_message>
new data, new labels, new heads
</commit_message>
<xml_diff>
--- a/docs/datasets_and_tasks.xlsx
+++ b/docs/datasets_and_tasks.xlsx
@@ -14,10 +14,10 @@
     <sheet name="Notes" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Datasets'!$A$1:$O$66</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Eval tasks'!$A$1:$S$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Datasets'!$A$1:$O$70</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Eval tasks'!$A$1:$S$70</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Training labels'!$A$1:$H$76</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Notes'!$A$1:$B$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Notes'!$A$1:$B$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -515,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:L20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -544,6 +544,9 @@
       <c r="G1" s="2" t="n"/>
       <c r="H1" s="2" t="n"/>
       <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+      <c r="L1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -558,35 +561,50 @@
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
+          <t>In store, not indexed</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Prep running</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
           <t>In pool, not prepared</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="F2" s="3" t="inlineStr">
         <is>
           <t>Access granted</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Public download</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>Apply</t>
         </is>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t>Candidate</t>
         </is>
       </c>
-      <c r="H2" s="3" t="inlineStr">
+      <c r="J2" s="3" t="inlineStr">
         <is>
           <t>Unidentified</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>Deleted</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -599,35 +617,47 @@
         </is>
       </c>
       <c r="B3" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A3,Datasets!$E$2:$E$66,B$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A3,Datasets!$E$2:$E$70,B$2)</f>
         <v/>
       </c>
       <c r="C3" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A3,Datasets!$E$2:$E$66,C$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A3,Datasets!$E$2:$E$70,C$2)</f>
         <v/>
       </c>
       <c r="D3" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A3,Datasets!$E$2:$E$66,D$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A3,Datasets!$E$2:$E$70,D$2)</f>
         <v/>
       </c>
       <c r="E3" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A3,Datasets!$E$2:$E$66,E$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A3,Datasets!$E$2:$E$70,E$2)</f>
         <v/>
       </c>
       <c r="F3" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A3,Datasets!$E$2:$E$66,F$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A3,Datasets!$E$2:$E$70,F$2)</f>
         <v/>
       </c>
       <c r="G3" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A3,Datasets!$E$2:$E$66,G$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A3,Datasets!$E$2:$E$70,G$2)</f>
         <v/>
       </c>
       <c r="H3" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A3,Datasets!$E$2:$E$66,H$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A3,Datasets!$E$2:$E$70,H$2)</f>
         <v/>
       </c>
       <c r="I3" s="2">
-        <f>SUM(B3:H3)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A3,Datasets!$E$2:$E$70,I$2)</f>
+        <v/>
+      </c>
+      <c r="J3" s="2">
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A3,Datasets!$E$2:$E$70,J$2)</f>
+        <v/>
+      </c>
+      <c r="K3" s="2">
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A3,Datasets!$E$2:$E$70,K$2)</f>
+        <v/>
+      </c>
+      <c r="L3" s="2">
+        <f>SUM(B3:K3)</f>
         <v/>
       </c>
     </row>
@@ -638,35 +668,47 @@
         </is>
       </c>
       <c r="B4" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A4,Datasets!$E$2:$E$66,B$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A4,Datasets!$E$2:$E$70,B$2)</f>
         <v/>
       </c>
       <c r="C4" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A4,Datasets!$E$2:$E$66,C$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A4,Datasets!$E$2:$E$70,C$2)</f>
         <v/>
       </c>
       <c r="D4" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A4,Datasets!$E$2:$E$66,D$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A4,Datasets!$E$2:$E$70,D$2)</f>
         <v/>
       </c>
       <c r="E4" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A4,Datasets!$E$2:$E$66,E$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A4,Datasets!$E$2:$E$70,E$2)</f>
         <v/>
       </c>
       <c r="F4" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A4,Datasets!$E$2:$E$66,F$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A4,Datasets!$E$2:$E$70,F$2)</f>
         <v/>
       </c>
       <c r="G4" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A4,Datasets!$E$2:$E$66,G$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A4,Datasets!$E$2:$E$70,G$2)</f>
         <v/>
       </c>
       <c r="H4" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A4,Datasets!$E$2:$E$66,H$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A4,Datasets!$E$2:$E$70,H$2)</f>
         <v/>
       </c>
       <c r="I4" s="2">
-        <f>SUM(B4:H4)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A4,Datasets!$E$2:$E$70,I$2)</f>
+        <v/>
+      </c>
+      <c r="J4" s="2">
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A4,Datasets!$E$2:$E$70,J$2)</f>
+        <v/>
+      </c>
+      <c r="K4" s="2">
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A4,Datasets!$E$2:$E$70,K$2)</f>
+        <v/>
+      </c>
+      <c r="L4" s="2">
+        <f>SUM(B4:K4)</f>
         <v/>
       </c>
     </row>
@@ -677,35 +719,47 @@
         </is>
       </c>
       <c r="B5" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A5,Datasets!$E$2:$E$66,B$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A5,Datasets!$E$2:$E$70,B$2)</f>
         <v/>
       </c>
       <c r="C5" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A5,Datasets!$E$2:$E$66,C$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A5,Datasets!$E$2:$E$70,C$2)</f>
         <v/>
       </c>
       <c r="D5" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A5,Datasets!$E$2:$E$66,D$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A5,Datasets!$E$2:$E$70,D$2)</f>
         <v/>
       </c>
       <c r="E5" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A5,Datasets!$E$2:$E$66,E$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A5,Datasets!$E$2:$E$70,E$2)</f>
         <v/>
       </c>
       <c r="F5" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A5,Datasets!$E$2:$E$66,F$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A5,Datasets!$E$2:$E$70,F$2)</f>
         <v/>
       </c>
       <c r="G5" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A5,Datasets!$E$2:$E$66,G$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A5,Datasets!$E$2:$E$70,G$2)</f>
         <v/>
       </c>
       <c r="H5" s="2">
-        <f>COUNTIFS(Datasets!$C$2:$C$66,$A5,Datasets!$E$2:$E$66,H$2)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A5,Datasets!$E$2:$E$70,H$2)</f>
         <v/>
       </c>
       <c r="I5" s="2">
-        <f>SUM(B5:H5)</f>
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A5,Datasets!$E$2:$E$70,I$2)</f>
+        <v/>
+      </c>
+      <c r="J5" s="2">
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A5,Datasets!$E$2:$E$70,J$2)</f>
+        <v/>
+      </c>
+      <c r="K5" s="2">
+        <f>COUNTIFS(Datasets!$C$2:$C$70,$A5,Datasets!$E$2:$E$70,K$2)</f>
+        <v/>
+      </c>
+      <c r="L5" s="2">
+        <f>SUM(B5:K5)</f>
         <v/>
       </c>
     </row>
@@ -745,6 +799,18 @@
       </c>
       <c r="I6" s="4">
         <f>SUM(I3:I5)</f>
+        <v/>
+      </c>
+      <c r="J6" s="4">
+        <f>SUM(J3:J5)</f>
+        <v/>
+      </c>
+      <c r="K6" s="4">
+        <f>SUM(K3:K5)</f>
+        <v/>
+      </c>
+      <c r="L6" s="4">
+        <f>SUM(L3:L5)</f>
         <v/>
       </c>
     </row>
@@ -758,6 +824,9 @@
       <c r="G7" s="2" t="n"/>
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="n"/>
+      <c r="J7" s="2" t="n"/>
+      <c r="K7" s="2" t="n"/>
+      <c r="L7" s="2" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
@@ -773,6 +842,9 @@
       <c r="G8" s="2" t="n"/>
       <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="n"/>
+      <c r="J8" s="2" t="n"/>
+      <c r="K8" s="2" t="n"/>
+      <c r="L8" s="2" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -804,6 +876,9 @@
       <c r="G9" s="2" t="n"/>
       <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="n"/>
+      <c r="J9" s="2" t="n"/>
+      <c r="K9" s="2" t="n"/>
+      <c r="L9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -812,25 +887,28 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>SUMIFS(Datasets!$F$2:$F$66,Datasets!$C$2:$C$66,$A10)</f>
+        <f>SUMIFS(Datasets!$F$2:$F$70,Datasets!$C$2:$C$70,$A10)</f>
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>SUMIFS(Datasets!$G$2:$G$66,Datasets!$C$2:$C$66,$A10)</f>
+        <f>SUMIFS(Datasets!$G$2:$G$70,Datasets!$C$2:$C$70,$A10)</f>
         <v/>
       </c>
       <c r="D10" s="5">
-        <f>SUMIFS(Datasets!$H$2:$H$66,Datasets!$C$2:$C$66,$A10)</f>
+        <f>SUMIFS(Datasets!$H$2:$H$70,Datasets!$C$2:$C$70,$A10)</f>
         <v/>
       </c>
       <c r="E10" s="5">
-        <f>SUMIFS(Datasets!$I$2:$I$66,Datasets!$C$2:$C$66,$A10)</f>
+        <f>SUMIFS(Datasets!$I$2:$I$70,Datasets!$C$2:$C$70,$A10)</f>
         <v/>
       </c>
       <c r="F10" s="2" t="n"/>
       <c r="G10" s="2" t="n"/>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
+      <c r="J10" s="2" t="n"/>
+      <c r="K10" s="2" t="n"/>
+      <c r="L10" s="2" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -839,25 +917,28 @@
         </is>
       </c>
       <c r="B11" s="5">
-        <f>SUMIFS(Datasets!$F$2:$F$66,Datasets!$C$2:$C$66,$A11)</f>
+        <f>SUMIFS(Datasets!$F$2:$F$70,Datasets!$C$2:$C$70,$A11)</f>
         <v/>
       </c>
       <c r="C11" s="5">
-        <f>SUMIFS(Datasets!$G$2:$G$66,Datasets!$C$2:$C$66,$A11)</f>
+        <f>SUMIFS(Datasets!$G$2:$G$70,Datasets!$C$2:$C$70,$A11)</f>
         <v/>
       </c>
       <c r="D11" s="5">
-        <f>SUMIFS(Datasets!$H$2:$H$66,Datasets!$C$2:$C$66,$A11)</f>
+        <f>SUMIFS(Datasets!$H$2:$H$70,Datasets!$C$2:$C$70,$A11)</f>
         <v/>
       </c>
       <c r="E11" s="5">
-        <f>SUMIFS(Datasets!$I$2:$I$66,Datasets!$C$2:$C$66,$A11)</f>
+        <f>SUMIFS(Datasets!$I$2:$I$70,Datasets!$C$2:$C$70,$A11)</f>
         <v/>
       </c>
       <c r="F11" s="2" t="n"/>
       <c r="G11" s="2" t="n"/>
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
+      <c r="J11" s="2" t="n"/>
+      <c r="K11" s="2" t="n"/>
+      <c r="L11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -885,6 +966,9 @@
       <c r="G12" s="4" t="n"/>
       <c r="H12" s="4" t="n"/>
       <c r="I12" s="4" t="n"/>
+      <c r="J12" s="4" t="n"/>
+      <c r="K12" s="4" t="n"/>
+      <c r="L12" s="4" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n"/>
@@ -896,6 +980,9 @@
       <c r="G13" s="2" t="n"/>
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="n"/>
+      <c r="J13" s="2" t="n"/>
+      <c r="K13" s="2" t="n"/>
+      <c r="L13" s="2" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="1" t="inlineStr">
@@ -911,6 +998,9 @@
       <c r="G14" s="2" t="n"/>
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="n"/>
+      <c r="J14" s="2" t="n"/>
+      <c r="K14" s="2" t="n"/>
+      <c r="L14" s="2" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -942,6 +1032,9 @@
       <c r="G15" s="2" t="n"/>
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="n"/>
+      <c r="J15" s="2" t="n"/>
+      <c r="K15" s="2" t="n"/>
+      <c r="L15" s="2" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -950,15 +1043,15 @@
         </is>
       </c>
       <c r="B16" s="2">
-        <f>COUNTIFS('Eval tasks'!$J$2:$J$68,"Benchmark v2",'Eval tasks'!$C$2:$C$68,B$15)</f>
+        <f>COUNTIFS('Eval tasks'!$J$2:$J$70,"Benchmark v2",'Eval tasks'!$C$2:$C$70,B$15)</f>
         <v/>
       </c>
       <c r="C16" s="2">
-        <f>COUNTIFS('Eval tasks'!$J$2:$J$68,"Benchmark v2",'Eval tasks'!$C$2:$C$68,C$15)</f>
+        <f>COUNTIFS('Eval tasks'!$J$2:$J$70,"Benchmark v2",'Eval tasks'!$C$2:$C$70,C$15)</f>
         <v/>
       </c>
       <c r="D16" s="2">
-        <f>COUNTIFS('Eval tasks'!$J$2:$J$68,"Benchmark v2",'Eval tasks'!$C$2:$C$68,D$15)</f>
+        <f>COUNTIFS('Eval tasks'!$J$2:$J$70,"Benchmark v2",'Eval tasks'!$C$2:$C$70,D$15)</f>
         <v/>
       </c>
       <c r="E16" s="2">
@@ -969,6 +1062,9 @@
       <c r="G16" s="2" t="n"/>
       <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="n"/>
+      <c r="J16" s="2" t="n"/>
+      <c r="K16" s="2" t="n"/>
+      <c r="L16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -977,15 +1073,15 @@
         </is>
       </c>
       <c r="B17" s="2">
-        <f>COUNTIFS('Eval tasks'!$J$2:$J$68,"Benchmark v2 (seg)",'Eval tasks'!$C$2:$C$68,B$15)</f>
+        <f>COUNTIFS('Eval tasks'!$J$2:$J$70,"Benchmark v2 (seg)",'Eval tasks'!$C$2:$C$70,B$15)</f>
         <v/>
       </c>
       <c r="C17" s="2">
-        <f>COUNTIFS('Eval tasks'!$J$2:$J$68,"Benchmark v2 (seg)",'Eval tasks'!$C$2:$C$68,C$15)</f>
+        <f>COUNTIFS('Eval tasks'!$J$2:$J$70,"Benchmark v2 (seg)",'Eval tasks'!$C$2:$C$70,C$15)</f>
         <v/>
       </c>
       <c r="D17" s="2">
-        <f>COUNTIFS('Eval tasks'!$J$2:$J$68,"Benchmark v2 (seg)",'Eval tasks'!$C$2:$C$68,D$15)</f>
+        <f>COUNTIFS('Eval tasks'!$J$2:$J$70,"Benchmark v2 (seg)",'Eval tasks'!$C$2:$C$70,D$15)</f>
         <v/>
       </c>
       <c r="E17" s="2">
@@ -996,6 +1092,9 @@
       <c r="G17" s="2" t="n"/>
       <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="n"/>
+      <c r="J17" s="2" t="n"/>
+      <c r="K17" s="2" t="n"/>
+      <c r="L17" s="2" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1004,15 +1103,15 @@
         </is>
       </c>
       <c r="B18" s="2">
-        <f>COUNTIFS('Eval tasks'!$J$2:$J$68,"Suite only*",'Eval tasks'!$C$2:$C$68,B$15)</f>
+        <f>COUNTIFS('Eval tasks'!$J$2:$J$70,"Suite only*",'Eval tasks'!$C$2:$C$70,B$15)</f>
         <v/>
       </c>
       <c r="C18" s="2">
-        <f>COUNTIFS('Eval tasks'!$J$2:$J$68,"Suite only*",'Eval tasks'!$C$2:$C$68,C$15)</f>
+        <f>COUNTIFS('Eval tasks'!$J$2:$J$70,"Suite only*",'Eval tasks'!$C$2:$C$70,C$15)</f>
         <v/>
       </c>
       <c r="D18" s="2">
-        <f>COUNTIFS('Eval tasks'!$J$2:$J$68,"Suite only*",'Eval tasks'!$C$2:$C$68,D$15)</f>
+        <f>COUNTIFS('Eval tasks'!$J$2:$J$70,"Suite only*",'Eval tasks'!$C$2:$C$70,D$15)</f>
         <v/>
       </c>
       <c r="E18" s="2">
@@ -1023,6 +1122,9 @@
       <c r="G18" s="2" t="n"/>
       <c r="H18" s="2" t="n"/>
       <c r="I18" s="2" t="n"/>
+      <c r="J18" s="2" t="n"/>
+      <c r="K18" s="2" t="n"/>
+      <c r="L18" s="2" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1031,15 +1133,15 @@
         </is>
       </c>
       <c r="B19" s="2">
-        <f>COUNTIFS('Eval tasks'!$J$2:$J$68,"Planned*",'Eval tasks'!$C$2:$C$68,B$15)</f>
+        <f>COUNTIFS('Eval tasks'!$J$2:$J$70,"Planned*",'Eval tasks'!$C$2:$C$70,B$15)</f>
         <v/>
       </c>
       <c r="C19" s="2">
-        <f>COUNTIFS('Eval tasks'!$J$2:$J$68,"Planned*",'Eval tasks'!$C$2:$C$68,C$15)</f>
+        <f>COUNTIFS('Eval tasks'!$J$2:$J$70,"Planned*",'Eval tasks'!$C$2:$C$70,C$15)</f>
         <v/>
       </c>
       <c r="D19" s="2">
-        <f>COUNTIFS('Eval tasks'!$J$2:$J$68,"Planned*",'Eval tasks'!$C$2:$C$68,D$15)</f>
+        <f>COUNTIFS('Eval tasks'!$J$2:$J$70,"Planned*",'Eval tasks'!$C$2:$C$70,D$15)</f>
         <v/>
       </c>
       <c r="E19" s="2">
@@ -1050,6 +1152,9 @@
       <c r="G19" s="2" t="n"/>
       <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="n"/>
+      <c r="J19" s="2" t="n"/>
+      <c r="K19" s="2" t="n"/>
+      <c r="L19" s="2" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
@@ -1077,6 +1182,9 @@
       <c r="G20" s="4" t="n"/>
       <c r="H20" s="4" t="n"/>
       <c r="I20" s="4" t="n"/>
+      <c r="J20" s="4" t="n"/>
+      <c r="K20" s="4" t="n"/>
+      <c r="L20" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1089,7 +1197,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O66"/>
+  <dimension ref="A1:O70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1642,7 +1750,7 @@
       </c>
       <c r="O9" s="7" t="inlineStr">
         <is>
-          <t>TCGA subset carries IDH / grade / survival labels (gli_* tasks). UCSF-PDGM and UPENN-GBM patients overlap BraTS 2021.</t>
+          <t>TCGA subset (98 GBM + 65 LGG patients) carries IDH / grade / survival labels (gli_* tasks). UCSF-PDGM and UPENN-GBM patients overlap BraTS 2021 (shared dedup_key).</t>
         </is>
       </c>
     </row>
@@ -1942,12 +2050,12 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>OASIS-1</t>
+          <t>UCSF-PDGM (preoperative diffuse glioma)</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>oasis1</t>
+          <t>ucsf_pdgm</t>
         </is>
       </c>
       <c r="C15" s="7" t="inlineStr">
@@ -1957,7 +2065,7 @@
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>t1 (436)</t>
+          <t>t1c (501), t1 (501), flair (501), t2 (501)</t>
         </is>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -1966,49 +2074,45 @@
         </is>
       </c>
       <c r="F15" s="8" t="n">
-        <v>416</v>
+        <v>495</v>
       </c>
       <c r="G15" s="8" t="n">
-        <v>436</v>
+        <v>2004</v>
       </c>
       <c r="H15" s="8" t="n">
-        <v>307</v>
+        <v>0</v>
       </c>
       <c r="I15" s="8" t="n">
-        <v>73</v>
+        <v>380</v>
       </c>
       <c r="J15" s="7" t="inlineStr"/>
       <c r="K15" s="7" t="inlineStr">
         <is>
-          <t>oasis1_cdr, oasis1_age, oasis1_mmse</t>
-        </is>
-      </c>
-      <c r="L15" s="7" t="inlineStr">
-        <is>
-          <t>SynthSeg morphometry (31 tasks); brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; mmse</t>
-        </is>
-      </c>
+          <t>ucsf_survival_12m, ucsf_lgg, ucsf_idh, ucsf_mgmt</t>
+        </is>
+      </c>
+      <c r="L15" s="7" t="inlineStr"/>
       <c r="M15" s="7" t="inlineStr"/>
       <c r="N15" s="7" t="inlineStr">
         <is>
-          <t>oasis-brains.org</t>
+          <t>TCIA (CC BY 4.0), Aspera</t>
         </is>
       </c>
       <c r="O15" s="7" t="inlineStr">
         <is>
-          <t>Train split in SSL pool. Its 235 CDR-labelled subjects = BrainIAC's and BrainDINO's dementia cohort.</t>
+          <t>Held out (eval only). 501 patients x T1 / T1c / T2 / FLAIR, one registration per patient (re-prepped 2026-10-29). ~1/3 of patients are BraTS 2021 twins (shared dedup_key; pretrain_overlap flags them). Tumour labels stored in BraTS 2023 numbering (enhancing 4 -&gt; 3).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>BraTS-GoAT 2024</t>
+          <t>OASIS-1</t>
         </is>
       </c>
       <c r="B16" s="7" t="inlineStr">
         <is>
-          <t>brats_goat</t>
+          <t>oasis1</t>
         </is>
       </c>
       <c r="C16" s="7" t="inlineStr">
@@ -2018,7 +2122,7 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>t1c (369), t2 (369), flair (367), t1 (366)</t>
+          <t>t1 (436)</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
@@ -2027,41 +2131,49 @@
         </is>
       </c>
       <c r="F16" s="8" t="n">
-        <v>370</v>
+        <v>416</v>
       </c>
       <c r="G16" s="8" t="n">
-        <v>1471</v>
+        <v>436</v>
       </c>
       <c r="H16" s="8" t="n">
-        <v>1141</v>
+        <v>307</v>
       </c>
       <c r="I16" s="8" t="n">
-        <v>175</v>
+        <v>73</v>
       </c>
       <c r="J16" s="7" t="inlineStr"/>
-      <c r="K16" s="7" t="inlineStr"/>
+      <c r="K16" s="7" t="inlineStr">
+        <is>
+          <t>oasis1_cdr, oasis1_age, oasis1_mmse</t>
+        </is>
+      </c>
       <c r="L16" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); brain_asymmetry; brain_volume; intensity_asymmetry</t>
+          <t>SynthSeg morphometry (31 tasks); brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; mmse</t>
         </is>
       </c>
       <c r="M16" s="7" t="inlineStr"/>
       <c r="N16" s="7" t="inlineStr">
         <is>
-          <t>Synapse (BraTS)</t>
-        </is>
-      </c>
-      <c r="O16" s="7" t="inlineStr"/>
+          <t>oasis-brains.org</t>
+        </is>
+      </c>
+      <c r="O16" s="7" t="inlineStr">
+        <is>
+          <t>Train split in SSL pool. Its 235 CDR-labelled subjects = BrainIAC's and BrainDINO's dementia cohort.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="7" t="inlineStr">
         <is>
-          <t>ISLES 2022 (DWI / ADC / FLAIR)</t>
+          <t>BraTS-GoAT 2024</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>isles22</t>
+          <t>brats_goat</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
@@ -2071,7 +2183,7 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>adc (249), flair (249), dwi (248)</t>
+          <t>t1c (369), t2 (369), flair (367), t1 (366)</t>
         </is>
       </c>
       <c r="E17" s="7" t="inlineStr">
@@ -2080,28 +2192,28 @@
         </is>
       </c>
       <c r="F17" s="8" t="n">
-        <v>249</v>
+        <v>370</v>
       </c>
       <c r="G17" s="8" t="n">
-        <v>746</v>
+        <v>1471</v>
       </c>
       <c r="H17" s="8" t="n">
-        <v>0</v>
+        <v>1141</v>
       </c>
       <c r="I17" s="8" t="n">
-        <v>114</v>
+        <v>175</v>
       </c>
       <c r="J17" s="7" t="inlineStr"/>
-      <c r="K17" s="7" t="inlineStr">
-        <is>
-          <t>isles22 (seg)</t>
-        </is>
-      </c>
-      <c r="L17" s="7" t="inlineStr"/>
+      <c r="K17" s="7" t="inlineStr"/>
+      <c r="L17" s="7" t="inlineStr">
+        <is>
+          <t>SynthSeg morphometry (31 tasks); brain_asymmetry; brain_volume; intensity_asymmetry</t>
+        </is>
+      </c>
       <c r="M17" s="7" t="inlineStr"/>
       <c r="N17" s="7" t="inlineStr">
         <is>
-          <t>ISLES'22 (Zenodo)</t>
+          <t>Synapse (BraTS)</t>
         </is>
       </c>
       <c r="O17" s="7" t="inlineStr"/>
@@ -2109,12 +2221,12 @@
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>AOMIC PIOP2</t>
+          <t>ISLES 2022 (DWI / ADC / FLAIR)</t>
         </is>
       </c>
       <c r="B18" s="7" t="inlineStr">
         <is>
-          <t>piop2</t>
+          <t>isles22</t>
         </is>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -2124,7 +2236,7 @@
       </c>
       <c r="D18" s="7" t="inlineStr">
         <is>
-          <t>t1 (226)</t>
+          <t>adc (249), flair (249), dwi (248)</t>
         </is>
       </c>
       <c r="E18" s="7" t="inlineStr">
@@ -2133,49 +2245,41 @@
         </is>
       </c>
       <c r="F18" s="8" t="n">
-        <v>226</v>
+        <v>249</v>
       </c>
       <c r="G18" s="8" t="n">
-        <v>226</v>
+        <v>746</v>
       </c>
       <c r="H18" s="8" t="n">
-        <v>169</v>
+        <v>0</v>
       </c>
       <c r="I18" s="8" t="n">
-        <v>34</v>
+        <v>114</v>
       </c>
       <c r="J18" s="7" t="inlineStr"/>
       <c r="K18" s="7" t="inlineStr">
         <is>
-          <t>piop2_age</t>
-        </is>
-      </c>
-      <c r="L18" s="7" t="inlineStr">
-        <is>
-          <t>SynthSeg morphometry (31 tasks); brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry</t>
-        </is>
-      </c>
+          <t>isles22 (seg)</t>
+        </is>
+      </c>
+      <c r="L18" s="7" t="inlineStr"/>
       <c r="M18" s="7" t="inlineStr"/>
       <c r="N18" s="7" t="inlineStr">
         <is>
-          <t>OpenNeuro (AOMIC)</t>
-        </is>
-      </c>
-      <c r="O18" s="7" t="inlineStr">
-        <is>
-          <t>Ages 18-26 only.</t>
-        </is>
-      </c>
+          <t>ISLES'22 (Zenodo)</t>
+        </is>
+      </c>
+      <c r="O18" s="7" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="7" t="inlineStr">
         <is>
-          <t>AOMIC PIOP1</t>
+          <t>AOMIC PIOP2</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>piop1</t>
+          <t>piop2</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
@@ -2185,7 +2289,7 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>t1 (216)</t>
+          <t>t1 (226)</t>
         </is>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -2194,21 +2298,21 @@
         </is>
       </c>
       <c r="F19" s="8" t="n">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="G19" s="8" t="n">
-        <v>216</v>
+        <v>226</v>
       </c>
       <c r="H19" s="8" t="n">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="I19" s="8" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J19" s="7" t="inlineStr"/>
       <c r="K19" s="7" t="inlineStr">
         <is>
-          <t>piop1_age</t>
+          <t>piop2_age</t>
         </is>
       </c>
       <c r="L19" s="7" t="inlineStr">
@@ -2231,12 +2335,12 @@
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>WMH Segmentation Challenge 2017</t>
+          <t>AOMIC PIOP1</t>
         </is>
       </c>
       <c r="B20" s="7" t="inlineStr">
         <is>
-          <t>wmh</t>
+          <t>piop1</t>
         </is>
       </c>
       <c r="C20" s="7" t="inlineStr">
@@ -2246,7 +2350,7 @@
       </c>
       <c r="D20" s="7" t="inlineStr">
         <is>
-          <t>flair (170), t1 (170)</t>
+          <t>t1 (216)</t>
         </is>
       </c>
       <c r="E20" s="7" t="inlineStr">
@@ -2255,41 +2359,49 @@
         </is>
       </c>
       <c r="F20" s="8" t="n">
-        <v>170</v>
+        <v>216</v>
       </c>
       <c r="G20" s="8" t="n">
-        <v>340</v>
+        <v>216</v>
       </c>
       <c r="H20" s="8" t="n">
-        <v>0</v>
+        <v>162</v>
       </c>
       <c r="I20" s="8" t="n">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="J20" s="7" t="inlineStr"/>
       <c r="K20" s="7" t="inlineStr">
         <is>
-          <t>wmh (seg)</t>
-        </is>
-      </c>
-      <c r="L20" s="7" t="inlineStr"/>
+          <t>piop1_age</t>
+        </is>
+      </c>
+      <c r="L20" s="7" t="inlineStr">
+        <is>
+          <t>SynthSeg morphometry (31 tasks); brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry</t>
+        </is>
+      </c>
       <c r="M20" s="7" t="inlineStr"/>
       <c r="N20" s="7" t="inlineStr">
         <is>
-          <t>WMH challenge (DataverseNL)</t>
-        </is>
-      </c>
-      <c r="O20" s="7" t="inlineStr"/>
+          <t>OpenNeuro (AOMIC)</t>
+        </is>
+      </c>
+      <c r="O20" s="7" t="inlineStr">
+        <is>
+          <t>Ages 18-26 only.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="7" t="inlineStr">
         <is>
-          <t>BrainMetShare (Stanford)</t>
+          <t>WMH Segmentation Challenge 2017</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>brainmetshare</t>
+          <t>wmh</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -2299,7 +2411,7 @@
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>t1c (312), t1 (156), flair (156)</t>
+          <t>flair (170), t1 (170)</t>
         </is>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -2308,24 +2420,28 @@
         </is>
       </c>
       <c r="F21" s="8" t="n">
-        <v>156</v>
+        <v>170</v>
       </c>
       <c r="G21" s="8" t="n">
-        <v>624</v>
+        <v>340</v>
       </c>
       <c r="H21" s="8" t="n">
         <v>0</v>
       </c>
       <c r="I21" s="8" t="n">
-        <v>92</v>
+        <v>52</v>
       </c>
       <c r="J21" s="7" t="inlineStr"/>
-      <c r="K21" s="7" t="inlineStr"/>
+      <c r="K21" s="7" t="inlineStr">
+        <is>
+          <t>wmh (seg)</t>
+        </is>
+      </c>
       <c r="L21" s="7" t="inlineStr"/>
       <c r="M21" s="7" t="inlineStr"/>
       <c r="N21" s="7" t="inlineStr">
         <is>
-          <t>Stanford AIMI</t>
+          <t>WMH challenge (DataverseNL)</t>
         </is>
       </c>
       <c r="O21" s="7" t="inlineStr"/>
@@ -2333,12 +2449,12 @@
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Pixar (OpenNeuro ds000228)</t>
+          <t>BrainMetShare (Stanford)</t>
         </is>
       </c>
       <c r="B22" s="7" t="inlineStr">
         <is>
-          <t>pixar</t>
+          <t>brainmetshare</t>
         </is>
       </c>
       <c r="C22" s="7" t="inlineStr">
@@ -2348,7 +2464,7 @@
       </c>
       <c r="D22" s="7" t="inlineStr">
         <is>
-          <t>t1 (155)</t>
+          <t>t1c (312), t1 (156), flair (156)</t>
         </is>
       </c>
       <c r="E22" s="7" t="inlineStr">
@@ -2357,32 +2473,24 @@
         </is>
       </c>
       <c r="F22" s="8" t="n">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="G22" s="8" t="n">
-        <v>155</v>
+        <v>624</v>
       </c>
       <c r="H22" s="8" t="n">
-        <v>116</v>
+        <v>0</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>23</v>
+        <v>92</v>
       </c>
       <c r="J22" s="7" t="inlineStr"/>
-      <c r="K22" s="7" t="inlineStr">
-        <is>
-          <t>pixar_age</t>
-        </is>
-      </c>
-      <c r="L22" s="7" t="inlineStr">
-        <is>
-          <t>SynthSeg morphometry (31 tasks); brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry</t>
-        </is>
-      </c>
+      <c r="K22" s="7" t="inlineStr"/>
+      <c r="L22" s="7" t="inlineStr"/>
       <c r="M22" s="7" t="inlineStr"/>
       <c r="N22" s="7" t="inlineStr">
         <is>
-          <t>OpenNeuro ds000228</t>
+          <t>Stanford AIMI</t>
         </is>
       </c>
       <c r="O22" s="7" t="inlineStr"/>
@@ -2390,12 +2498,12 @@
     <row r="23">
       <c r="A23" s="7" t="inlineStr">
         <is>
-          <t>OASIS-2 (longitudinal)</t>
+          <t>Pixar (OpenNeuro ds000228)</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>oasis2</t>
+          <t>pixar</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
@@ -2405,7 +2513,7 @@
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>t1 (373)</t>
+          <t>t1 (155)</t>
         </is>
       </c>
       <c r="E23" s="7" t="inlineStr">
@@ -2414,32 +2522,32 @@
         </is>
       </c>
       <c r="F23" s="8" t="n">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="G23" s="8" t="n">
-        <v>373</v>
+        <v>155</v>
       </c>
       <c r="H23" s="8" t="n">
-        <v>75</v>
+        <v>116</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>140</v>
+        <v>23</v>
       </c>
       <c r="J23" s="7" t="inlineStr"/>
       <c r="K23" s="7" t="inlineStr">
         <is>
-          <t>oasis2_cdr, oasis2_conversion, oasis2_mmse</t>
+          <t>pixar_age</t>
         </is>
       </c>
       <c r="L23" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; mmse</t>
+          <t>SynthSeg morphometry (31 tasks); brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry</t>
         </is>
       </c>
       <c r="M23" s="7" t="inlineStr"/>
       <c r="N23" s="7" t="inlineStr">
         <is>
-          <t>oasis-brains.org</t>
+          <t>OpenNeuro ds000228</t>
         </is>
       </c>
       <c r="O23" s="7" t="inlineStr"/>
@@ -2447,12 +2555,12 @@
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
-          <t>BraTS-PED 2023</t>
+          <t>OASIS-2 (longitudinal)</t>
         </is>
       </c>
       <c r="B24" s="7" t="inlineStr">
         <is>
-          <t>brats_ped</t>
+          <t>oasis2</t>
         </is>
       </c>
       <c r="C24" s="7" t="inlineStr">
@@ -2462,7 +2570,7 @@
       </c>
       <c r="D24" s="7" t="inlineStr">
         <is>
-          <t>t1c (143), t1 (143), flair (143), t2 (143)</t>
+          <t>t1 (373)</t>
         </is>
       </c>
       <c r="E24" s="7" t="inlineStr">
@@ -2471,32 +2579,32 @@
         </is>
       </c>
       <c r="F24" s="8" t="n">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>572</v>
+        <v>373</v>
       </c>
       <c r="H24" s="8" t="n">
-        <v>428</v>
+        <v>75</v>
       </c>
       <c r="I24" s="8" t="n">
-        <v>88</v>
+        <v>140</v>
       </c>
       <c r="J24" s="7" t="inlineStr"/>
       <c r="K24" s="7" t="inlineStr">
         <is>
-          <t>brats2023_ped (seg)</t>
+          <t>oasis2_cdr, oasis2_conversion, oasis2_mmse</t>
         </is>
       </c>
       <c r="L24" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); brain_asymmetry; brain_volume; intensity_asymmetry; tumor_type; tumor_volume; whole_tumor</t>
+          <t>SynthSeg morphometry (31 tasks); brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; mmse</t>
         </is>
       </c>
       <c r="M24" s="7" t="inlineStr"/>
       <c r="N24" s="7" t="inlineStr">
         <is>
-          <t>Synapse (BraTS)</t>
+          <t>oasis-brains.org</t>
         </is>
       </c>
       <c r="O24" s="7" t="inlineStr"/>
@@ -2504,12 +2612,12 @@
     <row r="25">
       <c r="A25" s="7" t="inlineStr">
         <is>
-          <t>MSD Task01 BrainTumour (non-BraTS remainder)</t>
+          <t>BraTS-PED 2023</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>msd_braintumor</t>
+          <t>brats_ped</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
@@ -2519,7 +2627,7 @@
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>t1 (115)</t>
+          <t>t1c (143), t1 (143), flair (143), t2 (143)</t>
         </is>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -2528,45 +2636,45 @@
         </is>
       </c>
       <c r="F25" s="8" t="n">
-        <v>115</v>
+        <v>143</v>
       </c>
       <c r="G25" s="8" t="n">
-        <v>115</v>
+        <v>572</v>
       </c>
       <c r="H25" s="8" t="n">
-        <v>0</v>
+        <v>428</v>
       </c>
       <c r="I25" s="8" t="n">
-        <v>16</v>
+        <v>88</v>
       </c>
       <c r="J25" s="7" t="inlineStr"/>
       <c r="K25" s="7" t="inlineStr">
         <is>
-          <t>msd</t>
-        </is>
-      </c>
-      <c r="L25" s="7" t="inlineStr"/>
+          <t>brats2023_ped (seg)</t>
+        </is>
+      </c>
+      <c r="L25" s="7" t="inlineStr">
+        <is>
+          <t>SynthSeg morphometry (31 tasks); brain_asymmetry; brain_volume; intensity_asymmetry; tumor_type; tumor_volume; whole_tumor</t>
+        </is>
+      </c>
       <c r="M25" s="7" t="inlineStr"/>
       <c r="N25" s="7" t="inlineStr">
         <is>
-          <t>Medical Segmentation Decathlon</t>
-        </is>
-      </c>
-      <c r="O25" s="7" t="inlineStr">
-        <is>
-          <t>MSD copies of BraTS 2017 cases were removed by content dedup; 115 remain.</t>
-        </is>
-      </c>
+          <t>Synapse (BraTS)</t>
+        </is>
+      </c>
+      <c r="O25" s="7" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="7" t="inlineStr">
         <is>
-          <t>MS3SEG</t>
+          <t>MSD Task01 BrainTumour (non-BraTS remainder)</t>
         </is>
       </c>
       <c r="B26" s="7" t="inlineStr">
         <is>
-          <t>ms3seg</t>
+          <t>msd_braintumor</t>
         </is>
       </c>
       <c r="C26" s="7" t="inlineStr">
@@ -2576,7 +2684,7 @@
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
-          <t>flair (100), t1 (100), t2 (100)</t>
+          <t>t1 (115)</t>
         </is>
       </c>
       <c r="E26" s="7" t="inlineStr">
@@ -2585,41 +2693,45 @@
         </is>
       </c>
       <c r="F26" s="8" t="n">
-        <v>100</v>
+        <v>115</v>
       </c>
       <c r="G26" s="8" t="n">
-        <v>300</v>
+        <v>115</v>
       </c>
       <c r="H26" s="8" t="n">
         <v>0</v>
       </c>
       <c r="I26" s="8" t="n">
-        <v>45</v>
+        <v>16</v>
       </c>
       <c r="J26" s="7" t="inlineStr"/>
       <c r="K26" s="7" t="inlineStr">
         <is>
-          <t>ms3seg_age, ms3seg_lesion_load, ms3seg (seg)</t>
+          <t>msd</t>
         </is>
       </c>
       <c r="L26" s="7" t="inlineStr"/>
       <c r="M26" s="7" t="inlineStr"/>
       <c r="N26" s="7" t="inlineStr">
         <is>
-          <t>figshare</t>
-        </is>
-      </c>
-      <c r="O26" s="7" t="inlineStr"/>
+          <t>Medical Segmentation Decathlon</t>
+        </is>
+      </c>
+      <c r="O26" s="7" t="inlineStr">
+        <is>
+          <t>MSD copies of BraTS 2017 cases were removed by content dedup; 115 remain.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
         <is>
-          <t>VALDO 2021 (small vessel disease)</t>
+          <t>MS3SEG</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>valdo</t>
+          <t>ms3seg</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
@@ -2629,7 +2741,7 @@
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>t1 (152), t2 (146), flair (80), t2s (72)</t>
+          <t>flair (100), t1 (100), t2 (100)</t>
         </is>
       </c>
       <c r="E27" s="7" t="inlineStr">
@@ -2638,45 +2750,41 @@
         </is>
       </c>
       <c r="F27" s="8" t="n">
-        <v>72</v>
+        <v>100</v>
       </c>
       <c r="G27" s="8" t="n">
-        <v>450</v>
+        <v>300</v>
       </c>
       <c r="H27" s="8" t="n">
         <v>0</v>
       </c>
       <c r="I27" s="8" t="n">
-        <v>63</v>
+        <v>45</v>
       </c>
       <c r="J27" s="7" t="inlineStr"/>
       <c r="K27" s="7" t="inlineStr">
         <is>
-          <t>valdo_epvs, valdo_cmb (seg), valdo_lacunes (seg)</t>
+          <t>ms3seg_age, ms3seg_lesion_load, ms3seg (seg)</t>
         </is>
       </c>
       <c r="L27" s="7" t="inlineStr"/>
       <c r="M27" s="7" t="inlineStr"/>
       <c r="N27" s="7" t="inlineStr">
         <is>
-          <t>VALDO (Zenodo)</t>
-        </is>
-      </c>
-      <c r="O27" s="7" t="inlineStr">
-        <is>
-          <t>Eval-only (pretrain=False).</t>
-        </is>
-      </c>
+          <t>figshare</t>
+        </is>
+      </c>
+      <c r="O27" s="7" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="7" t="inlineStr">
         <is>
-          <t>Healthy Brain Network (FOMO)</t>
+          <t>VALDO 2021 (small vessel disease)</t>
         </is>
       </c>
       <c r="B28" s="7" t="inlineStr">
         <is>
-          <t>fomo_hbn</t>
+          <t>valdo</t>
         </is>
       </c>
       <c r="C28" s="7" t="inlineStr">
@@ -2686,7 +2794,7 @@
       </c>
       <c r="D28" s="7" t="inlineStr">
         <is>
-          <t>t1 (3763), t2 (2806), pd (1183), flair (726)</t>
+          <t>t1 (152), t2 (146), flair (80), t2s (72)</t>
         </is>
       </c>
       <c r="E28" s="7" t="inlineStr">
@@ -2695,41 +2803,45 @@
         </is>
       </c>
       <c r="F28" s="8" t="n">
-        <v>3841</v>
+        <v>72</v>
       </c>
       <c r="G28" s="8" t="n">
-        <v>8478</v>
+        <v>450</v>
       </c>
       <c r="H28" s="8" t="n">
-        <v>5461</v>
+        <v>0</v>
       </c>
       <c r="I28" s="8" t="n">
-        <v>1280</v>
+        <v>63</v>
       </c>
       <c r="J28" s="7" t="inlineStr"/>
-      <c r="K28" s="7" t="inlineStr"/>
-      <c r="L28" s="7" t="inlineStr">
-        <is>
-          <t>SynthSeg morphometry (32 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
-        </is>
-      </c>
+      <c r="K28" s="7" t="inlineStr">
+        <is>
+          <t>valdo_epvs, valdo_cmb (seg), valdo_lacunes (seg)</t>
+        </is>
+      </c>
+      <c r="L28" s="7" t="inlineStr"/>
       <c r="M28" s="7" t="inlineStr"/>
       <c r="N28" s="7" t="inlineStr">
         <is>
-          <t>FOMO-260K compilation</t>
-        </is>
-      </c>
-      <c r="O28" s="7" t="inlineStr"/>
+          <t>VALDO (Zenodo)</t>
+        </is>
+      </c>
+      <c r="O28" s="7" t="inlineStr">
+        <is>
+          <t>Eval-only (pretrain=False).</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>CoRR (FOMO)</t>
+          <t>Healthy Brain Network (FOMO)</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
         <is>
-          <t>fomo_corr</t>
+          <t>fomo_hbn</t>
         </is>
       </c>
       <c r="C29" s="7" t="inlineStr">
@@ -2739,7 +2851,7 @@
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>t1 (2686)</t>
+          <t>t1 (3763), t2 (2806), pd (1183), flair (726)</t>
         </is>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -2748,22 +2860,22 @@
         </is>
       </c>
       <c r="F29" s="8" t="n">
-        <v>1472</v>
+        <v>3841</v>
       </c>
       <c r="G29" s="8" t="n">
-        <v>2686</v>
+        <v>8478</v>
       </c>
       <c r="H29" s="8" t="n">
-        <v>1103</v>
+        <v>5461</v>
       </c>
       <c r="I29" s="8" t="n">
-        <v>398</v>
+        <v>1280</v>
       </c>
       <c r="J29" s="7" t="inlineStr"/>
       <c r="K29" s="7" t="inlineStr"/>
       <c r="L29" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
+          <t>SynthSeg morphometry (32 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
         </is>
       </c>
       <c r="M29" s="7" t="inlineStr"/>
@@ -2777,12 +2889,12 @@
     <row r="30">
       <c r="A30" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO)</t>
+          <t>CoRR (FOMO)</t>
         </is>
       </c>
       <c r="B30" s="7" t="inlineStr">
         <is>
-          <t>fomo_yale_mets</t>
+          <t>fomo_corr</t>
         </is>
       </c>
       <c r="C30" s="7" t="inlineStr">
@@ -2792,7 +2904,7 @@
       </c>
       <c r="D30" s="7" t="inlineStr">
         <is>
-          <t>flair (9076), t1c (8992), t1 (8235), t2 (7325), pd (53)</t>
+          <t>t1 (2686)</t>
         </is>
       </c>
       <c r="E30" s="7" t="inlineStr">
@@ -2801,22 +2913,22 @@
         </is>
       </c>
       <c r="F30" s="8" t="n">
-        <v>1430</v>
+        <v>1472</v>
       </c>
       <c r="G30" s="8" t="n">
-        <v>33681</v>
+        <v>2686</v>
       </c>
       <c r="H30" s="8" t="n">
-        <v>3972</v>
+        <v>1103</v>
       </c>
       <c r="I30" s="8" t="n">
-        <v>5194</v>
+        <v>398</v>
       </c>
       <c r="J30" s="7" t="inlineStr"/>
       <c r="K30" s="7" t="inlineStr"/>
       <c r="L30" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_volume; intensity_asymmetry; sex; tumor_type</t>
+          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
         </is>
       </c>
       <c r="M30" s="7" t="inlineStr"/>
@@ -2830,12 +2942,12 @@
     <row r="31">
       <c r="A31" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO)</t>
+          <t>Yale brain metastases (FOMO)</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>fomo_nki</t>
+          <t>fomo_yale_mets</t>
         </is>
       </c>
       <c r="C31" s="7" t="inlineStr">
@@ -2845,7 +2957,7 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>t1 (2453), flair (2359), t2 (1136)</t>
+          <t>flair (9076), t1c (8992), t1 (8235), t2 (7325), pd (53)</t>
         </is>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -2854,22 +2966,22 @@
         </is>
       </c>
       <c r="F31" s="8" t="n">
-        <v>1326</v>
+        <v>1430</v>
       </c>
       <c r="G31" s="8" t="n">
-        <v>5948</v>
+        <v>33681</v>
       </c>
       <c r="H31" s="8" t="n">
-        <v>2354</v>
+        <v>3972</v>
       </c>
       <c r="I31" s="8" t="n">
-        <v>907</v>
+        <v>5194</v>
       </c>
       <c r="J31" s="7" t="inlineStr"/>
       <c r="K31" s="7" t="inlineStr"/>
       <c r="L31" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (32 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
+          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_volume; intensity_asymmetry; sex; tumor_type</t>
         </is>
       </c>
       <c r="M31" s="7" t="inlineStr"/>
@@ -2883,12 +2995,12 @@
     <row r="32">
       <c r="A32" s="7" t="inlineStr">
         <is>
-          <t>Infant MRI (FOMO)</t>
+          <t>NKI-Rockland (FOMO)</t>
         </is>
       </c>
       <c r="B32" s="7" t="inlineStr">
         <is>
-          <t>fomo_infant</t>
+          <t>fomo_nki</t>
         </is>
       </c>
       <c r="C32" s="7" t="inlineStr">
@@ -2898,7 +3010,7 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>t2 (833), t1 (832)</t>
+          <t>t1 (2453), flair (2359), t2 (1136)</t>
         </is>
       </c>
       <c r="E32" s="7" t="inlineStr">
@@ -2907,22 +3019,22 @@
         </is>
       </c>
       <c r="F32" s="8" t="n">
-        <v>833</v>
+        <v>1326</v>
       </c>
       <c r="G32" s="8" t="n">
-        <v>1665</v>
+        <v>5948</v>
       </c>
       <c r="H32" s="8" t="n">
-        <v>1110</v>
+        <v>2354</v>
       </c>
       <c r="I32" s="8" t="n">
-        <v>250</v>
+        <v>907</v>
       </c>
       <c r="J32" s="7" t="inlineStr"/>
       <c r="K32" s="7" t="inlineStr"/>
       <c r="L32" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; infant_abnormal; intensity_asymmetry</t>
+          <t>SynthSeg morphometry (32 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
         </is>
       </c>
       <c r="M32" s="7" t="inlineStr"/>
@@ -2936,12 +3048,12 @@
     <row r="33">
       <c r="A33" s="7" t="inlineStr">
         <is>
-          <t>SLIM longitudinal (FOMO)</t>
+          <t>Infant MRI (FOMO)</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>fomo_slim</t>
+          <t>fomo_infant</t>
         </is>
       </c>
       <c r="C33" s="7" t="inlineStr">
@@ -2951,7 +3063,7 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>t1 (1037)</t>
+          <t>t2 (833), t1 (832)</t>
         </is>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -2960,22 +3072,22 @@
         </is>
       </c>
       <c r="F33" s="8" t="n">
-        <v>588</v>
+        <v>833</v>
       </c>
       <c r="G33" s="8" t="n">
-        <v>1037</v>
+        <v>1665</v>
       </c>
       <c r="H33" s="8" t="n">
-        <v>441</v>
+        <v>1110</v>
       </c>
       <c r="I33" s="8" t="n">
-        <v>154</v>
+        <v>250</v>
       </c>
       <c r="J33" s="7" t="inlineStr"/>
       <c r="K33" s="7" t="inlineStr"/>
       <c r="L33" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
+          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; infant_abnormal; intensity_asymmetry</t>
         </is>
       </c>
       <c r="M33" s="7" t="inlineStr"/>
@@ -2989,12 +3101,12 @@
     <row r="34">
       <c r="A34" s="7" t="inlineStr">
         <is>
-          <t>BrainLat (FOMO)</t>
+          <t>SLIM longitudinal (FOMO)</t>
         </is>
       </c>
       <c r="B34" s="7" t="inlineStr">
         <is>
-          <t>fomo_brainlat</t>
+          <t>fomo_slim</t>
         </is>
       </c>
       <c r="C34" s="7" t="inlineStr">
@@ -3004,7 +3116,7 @@
       </c>
       <c r="D34" s="7" t="inlineStr">
         <is>
-          <t>t1 (576), flair (45)</t>
+          <t>t1 (1037)</t>
         </is>
       </c>
       <c r="E34" s="7" t="inlineStr">
@@ -3013,22 +3125,22 @@
         </is>
       </c>
       <c r="F34" s="8" t="n">
-        <v>576</v>
+        <v>588</v>
       </c>
       <c r="G34" s="8" t="n">
-        <v>621</v>
+        <v>1037</v>
       </c>
       <c r="H34" s="8" t="n">
-        <v>462</v>
+        <v>441</v>
       </c>
       <c r="I34" s="8" t="n">
-        <v>95</v>
+        <v>154</v>
       </c>
       <c r="J34" s="7" t="inlineStr"/>
       <c r="K34" s="7" t="inlineStr"/>
       <c r="L34" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (32 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; neuro_diagnosis; parkinsons; sex</t>
+          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
         </is>
       </c>
       <c r="M34" s="7" t="inlineStr"/>
@@ -3042,12 +3154,12 @@
     <row r="35">
       <c r="A35" s="7" t="inlineStr">
         <is>
-          <t>FOMO cohort: wayne</t>
+          <t>BrainLat (FOMO)</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>fomo_wayne</t>
+          <t>fomo_brainlat</t>
         </is>
       </c>
       <c r="C35" s="7" t="inlineStr">
@@ -3057,7 +3169,7 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>t1 (610)</t>
+          <t>t1 (576), flair (45)</t>
         </is>
       </c>
       <c r="E35" s="7" t="inlineStr">
@@ -3066,22 +3178,22 @@
         </is>
       </c>
       <c r="F35" s="8" t="n">
-        <v>426</v>
+        <v>576</v>
       </c>
       <c r="G35" s="8" t="n">
-        <v>610</v>
+        <v>621</v>
       </c>
       <c r="H35" s="8" t="n">
-        <v>319</v>
+        <v>462</v>
       </c>
       <c r="I35" s="8" t="n">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="J35" s="7" t="inlineStr"/>
       <c r="K35" s="7" t="inlineStr"/>
       <c r="L35" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
+          <t>SynthSeg morphometry (32 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; neuro_diagnosis; parkinsons; sex</t>
         </is>
       </c>
       <c r="M35" s="7" t="inlineStr"/>
@@ -3095,12 +3207,12 @@
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
         <is>
-          <t>FOMO cohort: yale_highres</t>
+          <t>FOMO cohort: wayne</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>fomo_yale_highres</t>
+          <t>fomo_wayne</t>
         </is>
       </c>
       <c r="C36" s="7" t="inlineStr">
@@ -3110,7 +3222,7 @@
       </c>
       <c r="D36" s="7" t="inlineStr">
         <is>
-          <t>t1 (268)</t>
+          <t>t1 (610)</t>
         </is>
       </c>
       <c r="E36" s="7" t="inlineStr">
@@ -3119,16 +3231,16 @@
         </is>
       </c>
       <c r="F36" s="8" t="n">
-        <v>232</v>
+        <v>426</v>
       </c>
       <c r="G36" s="8" t="n">
-        <v>268</v>
+        <v>610</v>
       </c>
       <c r="H36" s="8" t="n">
-        <v>174</v>
+        <v>319</v>
       </c>
       <c r="I36" s="8" t="n">
-        <v>41</v>
+        <v>102</v>
       </c>
       <c r="J36" s="7" t="inlineStr"/>
       <c r="K36" s="7" t="inlineStr"/>
@@ -3148,12 +3260,12 @@
     <row r="37">
       <c r="A37" s="7" t="inlineStr">
         <is>
-          <t>M4Raw low-field (FOMO)</t>
+          <t>FOMO cohort: yale_highres</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>fomo_m4raw</t>
+          <t>fomo_yale_highres</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
@@ -3163,7 +3275,7 @@
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>flair (208), t1 (208), t2 (208)</t>
+          <t>t1 (268)</t>
         </is>
       </c>
       <c r="E37" s="7" t="inlineStr">
@@ -3172,22 +3284,22 @@
         </is>
       </c>
       <c r="F37" s="8" t="n">
-        <v>208</v>
+        <v>232</v>
       </c>
       <c r="G37" s="8" t="n">
-        <v>624</v>
+        <v>268</v>
       </c>
       <c r="H37" s="8" t="n">
-        <v>468</v>
+        <v>174</v>
       </c>
       <c r="I37" s="8" t="n">
-        <v>93</v>
+        <v>41</v>
       </c>
       <c r="J37" s="7" t="inlineStr"/>
       <c r="K37" s="7" t="inlineStr"/>
       <c r="L37" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (32 tasks); brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry</t>
+          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
         </is>
       </c>
       <c r="M37" s="7" t="inlineStr"/>
@@ -3201,12 +3313,12 @@
     <row r="38">
       <c r="A38" s="7" t="inlineStr">
         <is>
-          <t>Cuban Human Brain Mapping (FOMO)</t>
+          <t>M4Raw low-field (FOMO)</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>fomo_chbmp</t>
+          <t>fomo_m4raw</t>
         </is>
       </c>
       <c r="C38" s="7" t="inlineStr">
@@ -3216,7 +3328,7 @@
       </c>
       <c r="D38" s="7" t="inlineStr">
         <is>
-          <t>t1 (203)</t>
+          <t>flair (208), t1 (208), t2 (208)</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
@@ -3225,22 +3337,22 @@
         </is>
       </c>
       <c r="F38" s="8" t="n">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="G38" s="8" t="n">
-        <v>203</v>
+        <v>624</v>
       </c>
       <c r="H38" s="8" t="n">
-        <v>153</v>
+        <v>468</v>
       </c>
       <c r="I38" s="8" t="n">
-        <v>30</v>
+        <v>93</v>
       </c>
       <c r="J38" s="7" t="inlineStr"/>
       <c r="K38" s="7" t="inlineStr"/>
       <c r="L38" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
+          <t>SynthSeg morphometry (32 tasks); brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry</t>
         </is>
       </c>
       <c r="M38" s="7" t="inlineStr"/>
@@ -3254,12 +3366,12 @@
     <row r="39">
       <c r="A39" s="7" t="inlineStr">
         <is>
-          <t>FOMO cohort: beijing</t>
+          <t>Cuban Human Brain Mapping (FOMO)</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>fomo_beijing</t>
+          <t>fomo_chbmp</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
@@ -3269,7 +3381,7 @@
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>t1 (180)</t>
+          <t>t1 (203)</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
@@ -3278,22 +3390,22 @@
         </is>
       </c>
       <c r="F39" s="8" t="n">
-        <v>180</v>
+        <v>203</v>
       </c>
       <c r="G39" s="8" t="n">
-        <v>180</v>
+        <v>203</v>
       </c>
       <c r="H39" s="8" t="n">
-        <v>135</v>
+        <v>153</v>
       </c>
       <c r="I39" s="8" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J39" s="7" t="inlineStr"/>
       <c r="K39" s="7" t="inlineStr"/>
       <c r="L39" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
+          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
         </is>
       </c>
       <c r="M39" s="7" t="inlineStr"/>
@@ -3307,12 +3419,12 @@
     <row r="40">
       <c r="A40" s="7" t="inlineStr">
         <is>
-          <t>WAND (FOMO)</t>
+          <t>FOMO cohort: beijing</t>
         </is>
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>fomo_wand</t>
+          <t>fomo_beijing</t>
         </is>
       </c>
       <c r="C40" s="7" t="inlineStr">
@@ -3322,7 +3434,7 @@
       </c>
       <c r="D40" s="7" t="inlineStr">
         <is>
-          <t>t1 (656), t2 (170)</t>
+          <t>t1 (180)</t>
         </is>
       </c>
       <c r="E40" s="7" t="inlineStr">
@@ -3331,22 +3443,22 @@
         </is>
       </c>
       <c r="F40" s="8" t="n">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="G40" s="8" t="n">
-        <v>826</v>
+        <v>180</v>
       </c>
       <c r="H40" s="8" t="n">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="I40" s="8" t="n">
-        <v>129</v>
+        <v>27</v>
       </c>
       <c r="J40" s="7" t="inlineStr"/>
       <c r="K40" s="7" t="inlineStr"/>
       <c r="L40" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
+          <t>SynthSeg morphometry (31 tasks); brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
         </is>
       </c>
       <c r="M40" s="7" t="inlineStr"/>
@@ -3360,12 +3472,12 @@
     <row r="41">
       <c r="A41" s="7" t="inlineStr">
         <is>
-          <t>ACPI (FOMO)</t>
+          <t>WAND (FOMO)</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>fomo_acpi</t>
+          <t>fomo_wand</t>
         </is>
       </c>
       <c r="C41" s="7" t="inlineStr">
@@ -3375,7 +3487,7 @@
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>t1 (163)</t>
+          <t>t1 (656), t2 (170)</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -3384,22 +3496,22 @@
         </is>
       </c>
       <c r="F41" s="8" t="n">
-        <v>163</v>
+        <v>177</v>
       </c>
       <c r="G41" s="8" t="n">
-        <v>163</v>
+        <v>826</v>
       </c>
       <c r="H41" s="8" t="n">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="I41" s="8" t="n">
-        <v>24</v>
+        <v>129</v>
       </c>
       <c r="J41" s="7" t="inlineStr"/>
       <c r="K41" s="7" t="inlineStr"/>
       <c r="L41" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); adhd; age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
+          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
         </is>
       </c>
       <c r="M41" s="7" t="inlineStr"/>
@@ -3413,12 +3525,12 @@
     <row r="42">
       <c r="A42" s="7" t="inlineStr">
         <is>
-          <t>FOMO cohort: ageility</t>
+          <t>ACPI (FOMO)</t>
         </is>
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>fomo_ageility</t>
+          <t>fomo_acpi</t>
         </is>
       </c>
       <c r="C42" s="7" t="inlineStr">
@@ -3428,7 +3540,7 @@
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
-          <t>t1 (131)</t>
+          <t>t1 (163)</t>
         </is>
       </c>
       <c r="E42" s="7" t="inlineStr">
@@ -3437,22 +3549,22 @@
         </is>
       </c>
       <c r="F42" s="8" t="n">
-        <v>131</v>
+        <v>163</v>
       </c>
       <c r="G42" s="8" t="n">
-        <v>131</v>
+        <v>163</v>
       </c>
       <c r="H42" s="8" t="n">
-        <v>98</v>
+        <v>123</v>
       </c>
       <c r="I42" s="8" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="J42" s="7" t="inlineStr"/>
       <c r="K42" s="7" t="inlineStr"/>
       <c r="L42" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
+          <t>SynthSeg morphometry (31 tasks); adhd; age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
         </is>
       </c>
       <c r="M42" s="7" t="inlineStr"/>
@@ -3466,12 +3578,12 @@
     <row r="43">
       <c r="A43" s="7" t="inlineStr">
         <is>
-          <t>AHEAD 7T (FOMO)</t>
+          <t>FOMO cohort: ageility</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>fomo_ahead</t>
+          <t>fomo_ageility</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
@@ -3481,7 +3593,7 @@
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>t1 (105)</t>
+          <t>t1 (131)</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
@@ -3490,22 +3602,22 @@
         </is>
       </c>
       <c r="F43" s="8" t="n">
-        <v>105</v>
+        <v>131</v>
       </c>
       <c r="G43" s="8" t="n">
-        <v>105</v>
+        <v>131</v>
       </c>
       <c r="H43" s="8" t="n">
-        <v>79</v>
+        <v>98</v>
       </c>
       <c r="I43" s="8" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="J43" s="7" t="inlineStr"/>
       <c r="K43" s="7" t="inlineStr"/>
       <c r="L43" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (13 tasks); brain_mask; sex</t>
+          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
         </is>
       </c>
       <c r="M43" s="7" t="inlineStr"/>
@@ -3519,12 +3631,12 @@
     <row r="44">
       <c r="A44" s="7" t="inlineStr">
         <is>
-          <t>FOMO cohort: nigerian</t>
+          <t>AHEAD 7T (FOMO)</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>fomo_nigerian</t>
+          <t>fomo_ahead</t>
         </is>
       </c>
       <c r="C44" s="7" t="inlineStr">
@@ -3534,7 +3646,7 @@
       </c>
       <c r="D44" s="7" t="inlineStr">
         <is>
-          <t>t1 (110), t2 (96), flair (73)</t>
+          <t>t1 (105)</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
@@ -3543,22 +3655,22 @@
         </is>
       </c>
       <c r="F44" s="8" t="n">
-        <v>82</v>
+        <v>105</v>
       </c>
       <c r="G44" s="8" t="n">
-        <v>279</v>
+        <v>105</v>
       </c>
       <c r="H44" s="8" t="n">
-        <v>158</v>
+        <v>79</v>
       </c>
       <c r="I44" s="8" t="n">
-        <v>47</v>
+        <v>16</v>
       </c>
       <c r="J44" s="7" t="inlineStr"/>
       <c r="K44" s="7" t="inlineStr"/>
       <c r="L44" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (32 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
+          <t>SynthSeg morphometry (13 tasks); brain_mask; sex</t>
         </is>
       </c>
       <c r="M44" s="7" t="inlineStr"/>
@@ -3572,12 +3684,12 @@
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
         <is>
-          <t>FOMO cohort: abd</t>
+          <t>FOMO cohort: nigerian</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>fomo_abd</t>
+          <t>fomo_nigerian</t>
         </is>
       </c>
       <c r="C45" s="7" t="inlineStr">
@@ -3587,7 +3699,7 @@
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>t1 (96), t2 (79)</t>
+          <t>t1 (110), t2 (96), flair (73)</t>
         </is>
       </c>
       <c r="E45" s="7" t="inlineStr">
@@ -3596,22 +3708,22 @@
         </is>
       </c>
       <c r="F45" s="8" t="n">
-        <v>51</v>
+        <v>82</v>
       </c>
       <c r="G45" s="8" t="n">
-        <v>175</v>
+        <v>279</v>
       </c>
       <c r="H45" s="8" t="n">
-        <v>73</v>
+        <v>158</v>
       </c>
       <c r="I45" s="8" t="n">
-        <v>23</v>
+        <v>47</v>
       </c>
       <c r="J45" s="7" t="inlineStr"/>
       <c r="K45" s="7" t="inlineStr"/>
       <c r="L45" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry</t>
+          <t>SynthSeg morphometry (32 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
         </is>
       </c>
       <c r="M45" s="7" t="inlineStr"/>
@@ -3625,12 +3737,12 @@
     <row r="46">
       <c r="A46" s="7" t="inlineStr">
         <is>
-          <t>FOMO cohort: cunmet</t>
+          <t>FOMO cohort: abd</t>
         </is>
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>fomo_cunmet</t>
+          <t>fomo_abd</t>
         </is>
       </c>
       <c r="C46" s="7" t="inlineStr">
@@ -3640,7 +3752,7 @@
       </c>
       <c r="D46" s="7" t="inlineStr">
         <is>
-          <t>t1 (59)</t>
+          <t>t1 (96), t2 (79)</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
@@ -3652,19 +3764,19 @@
         <v>51</v>
       </c>
       <c r="G46" s="8" t="n">
-        <v>59</v>
+        <v>175</v>
       </c>
       <c r="H46" s="8" t="n">
-        <v>38</v>
+        <v>73</v>
       </c>
       <c r="I46" s="8" t="n">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="J46" s="7" t="inlineStr"/>
       <c r="K46" s="7" t="inlineStr"/>
       <c r="L46" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); adhd; age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
+          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry</t>
         </is>
       </c>
       <c r="M46" s="7" t="inlineStr"/>
@@ -3678,12 +3790,12 @@
     <row r="47">
       <c r="A47" s="7" t="inlineStr">
         <is>
-          <t>MICA-MICs (FOMO)</t>
+          <t>FOMO cohort: cunmet</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>fomo_mica</t>
+          <t>fomo_cunmet</t>
         </is>
       </c>
       <c r="C47" s="7" t="inlineStr">
@@ -3693,7 +3805,7 @@
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>t1 (50)</t>
+          <t>t1 (59)</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
@@ -3702,22 +3814,22 @@
         </is>
       </c>
       <c r="F47" s="8" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G47" s="8" t="n">
-        <v>50</v>
+        <v>59</v>
       </c>
       <c r="H47" s="8" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I47" s="8" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J47" s="7" t="inlineStr"/>
       <c r="K47" s="7" t="inlineStr"/>
       <c r="L47" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry</t>
+          <t>SynthSeg morphometry (31 tasks); adhd; age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
         </is>
       </c>
       <c r="M47" s="7" t="inlineStr"/>
@@ -3731,12 +3843,12 @@
     <row r="48">
       <c r="A48" s="7" t="inlineStr">
         <is>
-          <t>Tao Wu Parkinson's (FOMO)</t>
+          <t>MICA-MICs (FOMO)</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>fomo_taowu</t>
+          <t>fomo_mica</t>
         </is>
       </c>
       <c r="C48" s="7" t="inlineStr">
@@ -3746,7 +3858,7 @@
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>t1 (40)</t>
+          <t>t1 (50)</t>
         </is>
       </c>
       <c r="E48" s="7" t="inlineStr">
@@ -3755,22 +3867,22 @@
         </is>
       </c>
       <c r="F48" s="8" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="G48" s="8" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="H48" s="8" t="n">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="I48" s="8" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J48" s="7" t="inlineStr"/>
       <c r="K48" s="7" t="inlineStr"/>
       <c r="L48" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; parkinsons; sex</t>
+          <t>SynthSeg morphometry (31 tasks); brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry</t>
         </is>
       </c>
       <c r="M48" s="7" t="inlineStr"/>
@@ -3784,12 +3896,12 @@
     <row r="49">
       <c r="A49" s="7" t="inlineStr">
         <is>
-          <t>FOMO cohort: cleveland</t>
+          <t>Tao Wu Parkinson's (FOMO)</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>fomo_cleveland</t>
+          <t>fomo_taowu</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
@@ -3799,7 +3911,7 @@
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>t1 (31)</t>
+          <t>t1 (40)</t>
         </is>
       </c>
       <c r="E49" s="7" t="inlineStr">
@@ -3808,22 +3920,22 @@
         </is>
       </c>
       <c r="F49" s="8" t="n">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="G49" s="8" t="n">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="H49" s="8" t="n">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="I49" s="8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="J49" s="7" t="inlineStr"/>
       <c r="K49" s="7" t="inlineStr"/>
       <c r="L49" s="7" t="inlineStr">
         <is>
-          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
+          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; parkinsons; sex</t>
         </is>
       </c>
       <c r="M49" s="7" t="inlineStr"/>
@@ -3837,12 +3949,12 @@
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>FOMO cohort: hbnssi</t>
+          <t>FOMO cohort: cleveland</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>fomo_hbnssi</t>
+          <t>fomo_cleveland</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
@@ -3852,7 +3964,7 @@
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>t1 (167), t2 (12)</t>
+          <t>t1 (31)</t>
         </is>
       </c>
       <c r="E50" s="7" t="inlineStr">
@@ -3861,16 +3973,16 @@
         </is>
       </c>
       <c r="F50" s="8" t="n">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="G50" s="8" t="n">
-        <v>179</v>
+        <v>31</v>
       </c>
       <c r="H50" s="8" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="I50" s="8" t="n">
-        <v>28</v>
+        <v>5</v>
       </c>
       <c r="J50" s="7" t="inlineStr"/>
       <c r="K50" s="7" t="inlineStr"/>
@@ -3890,10 +4002,14 @@
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>ADNI</t>
-        </is>
-      </c>
-      <c r="B51" s="7" t="inlineStr"/>
+          <t>FOMO cohort: hbnssi</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>fomo_hbnssi</t>
+        </is>
+      </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
           <t>MRI</t>
@@ -3901,49 +4017,45 @@
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>T1 (MPRAGE / IR-SPGR), FLAIR, T2*, DWI, ...</t>
+          <t>t1 (167), t2 (12)</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>Access granted</t>
-        </is>
-      </c>
-      <c r="F51" s="8" t="n"/>
-      <c r="G51" s="8" t="n"/>
-      <c r="H51" s="8" t="n"/>
-      <c r="I51" s="8" t="n"/>
-      <c r="J51" s="7" t="inlineStr">
-        <is>
-          <t>~2,700 participants (ADNI-1/GO/2/3); ADNI-4 enrolling; repeated visits</t>
-        </is>
-      </c>
-      <c r="K51" s="7" t="inlineStr">
-        <is>
-          <t>CN vs AD; CN vs MCI; CN/MCI/AD; sMCI vs pMCI (36 mo); MMSE</t>
-        </is>
-      </c>
-      <c r="L51" s="7" t="inlineStr"/>
-      <c r="M51" s="7" t="inlineStr">
-        <is>
-          <t>LONI IDA application (granted)</t>
-        </is>
-      </c>
+          <t>In store</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="n">
+        <v>13</v>
+      </c>
+      <c r="G51" s="8" t="n">
+        <v>179</v>
+      </c>
+      <c r="H51" s="8" t="n">
+        <v>19</v>
+      </c>
+      <c r="I51" s="8" t="n">
+        <v>28</v>
+      </c>
+      <c r="J51" s="7" t="inlineStr"/>
+      <c r="K51" s="7" t="inlineStr"/>
+      <c r="L51" s="7" t="inlineStr">
+        <is>
+          <t>SynthSeg morphometry (31 tasks); age; brain_asymmetry; brain_mask; brain_volume; intensity_asymmetry; sex</t>
+        </is>
+      </c>
+      <c r="M51" s="7" t="inlineStr"/>
       <c r="N51" s="7" t="inlineStr">
         <is>
-          <t>ida.loni.usc.edu</t>
-        </is>
-      </c>
-      <c r="O51" s="7" t="inlineStr">
-        <is>
-          <t>Keep evaluation-only (out of SSL and multitask). Download job: jobs/download_adni.sbatch.</t>
-        </is>
-      </c>
+          <t>FOMO-260K compilation</t>
+        </is>
+      </c>
+      <c r="O51" s="7" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>PPMI</t>
+          <t>ADNI</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr"/>
@@ -3954,12 +4066,12 @@
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>T1 (baseline)</t>
+          <t>T1 (MPRAGE / IR-SPGR), FLAIR, T2*, DWI, ...</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>Apply</t>
+          <t>Access granted</t>
         </is>
       </c>
       <c r="F52" s="8" t="n"/>
@@ -3968,35 +4080,35 @@
       <c r="I52" s="8" t="n"/>
       <c r="J52" s="7" t="inlineStr">
         <is>
-          <t>BrainDINO used ~1,158 PD + ~283 controls</t>
+          <t>~2,700 participants (ADNI-1/GO/2/3); ADNI-4 enrolling; repeated visits</t>
         </is>
       </c>
       <c r="K52" s="7" t="inlineStr">
         <is>
-          <t>PD vs control</t>
+          <t>CN vs AD; CN vs MCI; CN/MCI/AD; sMCI vs pMCI (36 mo); MMSE</t>
         </is>
       </c>
       <c r="L52" s="7" t="inlineStr"/>
       <c r="M52" s="7" t="inlineStr">
         <is>
-          <t>PPMI data access application</t>
+          <t>LONI IDA application (granted)</t>
         </is>
       </c>
       <c r="N52" s="7" t="inlineStr">
         <is>
-          <t>ppmi-info.org (LONI IDA)</t>
+          <t>ida.loni.usc.edu</t>
         </is>
       </c>
       <c r="O52" s="7" t="inlineStr">
         <is>
-          <t>Proposal drafted earlier (research proposal doc).</t>
+          <t>Keep evaluation-only (out of SSL and multitask). Download job: jobs/download_adni.sbatch.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>UCSF-PDGM</t>
+          <t>PPMI</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr"/>
@@ -4007,12 +4119,12 @@
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>T1, T1c, T2, FLAIR, DWI, SWI, ASL</t>
+          <t>T1 (baseline)</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>Public download</t>
+          <t>Apply</t>
         </is>
       </c>
       <c r="F53" s="8" t="n"/>
@@ -4021,28 +4133,28 @@
       <c r="I53" s="8" t="n"/>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>~500 adult diffuse gliomas</t>
+          <t>BrainDINO used ~1,158 PD + ~283 controls</t>
         </is>
       </c>
       <c r="K53" s="7" t="inlineStr">
         <is>
-          <t>IDH status; WHO grade; MGMT; overall survival</t>
+          <t>PD vs control</t>
         </is>
       </c>
       <c r="L53" s="7" t="inlineStr"/>
       <c r="M53" s="7" t="inlineStr">
         <is>
-          <t>TCIA, CC BY 4.0</t>
+          <t>PPMI data access application</t>
         </is>
       </c>
       <c r="N53" s="7" t="inlineStr">
         <is>
-          <t>doi:10.7937/tcia.bdgf-8v37</t>
+          <t>ppmi-info.org (LONI IDA)</t>
         </is>
       </c>
       <c r="O53" s="7" t="inlineStr">
         <is>
-          <t>Many patients also in BraTS 2021 (used in SSL / tumour training): dedup + hold-out needed.</t>
+          <t>Proposal drafted earlier (research proposal doc).</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4164,11 @@
           <t>UPENN-GBM</t>
         </is>
       </c>
-      <c r="B54" s="7" t="inlineStr"/>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>upenn_gbm</t>
+        </is>
+      </c>
       <c r="C54" s="7" t="inlineStr">
         <is>
           <t>MRI</t>
@@ -4060,21 +4176,27 @@
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>T1, T1c, T2, FLAIR (+ DTI, DSC)</t>
+          <t>T1, T1c, T2, FLAIR (671 each)</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>Public download</t>
-        </is>
-      </c>
-      <c r="F54" s="8" t="n"/>
-      <c r="G54" s="8" t="n"/>
-      <c r="H54" s="8" t="n"/>
+          <t>In store, not indexed</t>
+        </is>
+      </c>
+      <c r="F54" s="8" t="n">
+        <v>630</v>
+      </c>
+      <c r="G54" s="8" t="n">
+        <v>2684</v>
+      </c>
+      <c r="H54" s="8" t="n">
+        <v>0</v>
+      </c>
       <c r="I54" s="8" t="n"/>
       <c r="J54" s="7" t="inlineStr">
         <is>
-          <t>~630 de novo glioblastoma patients</t>
+          <t>671 scans of 630 de novo glioblastoma patients</t>
         </is>
       </c>
       <c r="K54" s="7" t="inlineStr">
@@ -4085,7 +4207,7 @@
       <c r="L54" s="7" t="inlineStr"/>
       <c r="M54" s="7" t="inlineStr">
         <is>
-          <t>TCIA, CC BY 4.0</t>
+          <t>TCIA, CC BY 4.0 (Aspera)</t>
         </is>
       </c>
       <c r="N54" s="7" t="inlineStr">
@@ -4095,7 +4217,7 @@
       </c>
       <c r="O54" s="7" t="inlineStr">
         <is>
-          <t>Overlaps BraTS 2021: dedup + hold-out needed.</t>
+          <t>Prepped 2026-10-29 (2,684 volumes, all QC ok, one registration per scan); held out. UPenn is BraTS site 1: BraTS twins to be content-matched before indexing. 611 scans ship a tumour segmentation (labels stored 1/2/3). IDH: only 19 mutant (no IDH task).</t>
         </is>
       </c>
     </row>
@@ -4485,7 +4607,7 @@
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>In pool, not prepared</t>
+          <t>Deleted</t>
         </is>
       </c>
       <c r="F62" s="8" t="n"/>
@@ -4504,14 +4626,10 @@
           <t>Redivis</t>
         </is>
       </c>
-      <c r="N62" s="7" t="inlineStr">
-        <is>
-          <t>pool/datasets/sinoct</t>
-        </is>
-      </c>
+      <c r="N62" s="7" t="inlineStr"/>
       <c r="O62" s="7" t="inlineStr">
         <is>
-          <t>No RSNA-ICH overlap (pixel-fingerprint blocklist, brain/datasets/download_sinoct.py).</t>
+          <t>Downloaded, then deleted (2026-10-28).</t>
         </is>
       </c>
     </row>
@@ -4533,28 +4651,32 @@
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>CTA, MRA, T1 post, T2</t>
+          <t>CTA 1,808, MRA 1,252, T2 983, T1 post 305</t>
         </is>
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>In pool, not prepared</t>
+          <t>Prep running</t>
         </is>
       </c>
       <c r="F63" s="8" t="n"/>
       <c r="G63" s="8" t="n"/>
       <c r="H63" s="8" t="n"/>
       <c r="I63" s="8" t="n"/>
-      <c r="J63" s="7" t="inlineStr"/>
+      <c r="J63" s="7" t="inlineStr">
+        <is>
+          <t>4,348 series</t>
+        </is>
+      </c>
       <c r="K63" s="7" t="inlineStr">
         <is>
-          <t>Aneurysm presence; location (vessel segments)</t>
+          <t>Aneurysm presence; location (13 vessel segments)</t>
         </is>
       </c>
       <c r="L63" s="7" t="inlineStr"/>
       <c r="M63" s="7" t="inlineStr">
         <is>
-          <t>Kaggle (non-commercial, no redistribution)</t>
+          <t>MIRA dataset 7 (non-commercial, no redistribution)</t>
         </is>
       </c>
       <c r="N63" s="7" t="inlineStr">
@@ -4562,12 +4684,16 @@
           <t>pool/datasets/rsna_ica</t>
         </is>
       </c>
-      <c r="O63" s="7" t="inlineStr"/>
+      <c r="O63" s="7" t="inlineStr">
+        <is>
+          <t>Full prep started 2026-10-29 (4 shards). Mis-tagged CTA rescale headers undone (dicom.fix_ct_rescale): pilot CTA 27/30 ok. 2,254 aneurysm points + 178 vessel segmentations not yet mapped to the grid.</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>APIS</t>
+          <t>TCGA-GBM</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr"/>
@@ -4578,45 +4704,49 @@
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>Paired NCCT + ADC</t>
+          <t>Mixed clinical MR (T1, T1c, T2, FLAIR, ...); some CT</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr">
         <is>
-          <t>Candidate</t>
+          <t>Apply</t>
         </is>
       </c>
       <c r="F64" s="8" t="n"/>
       <c r="G64" s="8" t="n"/>
       <c r="H64" s="8" t="n"/>
       <c r="I64" s="8" t="n"/>
-      <c r="J64" s="7" t="inlineStr"/>
+      <c r="J64" s="7" t="inlineStr">
+        <is>
+          <t>262 patients, 575 studies, 5,412 series (74 GB)</t>
+        </is>
+      </c>
       <c r="K64" s="7" t="inlineStr">
         <is>
-          <t>Ischemic lesion segmentation (CT and MRI)</t>
+          <t>Glioblastoma survival; tumour on CT</t>
         </is>
       </c>
       <c r="L64" s="7" t="inlineStr"/>
       <c r="M64" s="7" t="inlineStr">
         <is>
-          <t>Challenge registration</t>
+          <t>TCIA Restricted License (signed, per collection)</t>
         </is>
       </c>
       <c r="N64" s="7" t="inlineStr">
         <is>
-          <t>APIS challenge</t>
+          <t>doi:10.7937/K9/TCIA.2016.RNYFUYE9</t>
         </is>
       </c>
       <c r="O64" s="7" t="inlineStr">
         <is>
-          <t>Paired CT / MRI of the same stroke: a direct modality-agnosticism test.</t>
+          <t>98 patients' pre-op MRI already in the store via BraTS. Survival / IDH for all from TCGA (cBioPortal). Heterogeneous DICOM; sequence identification needed. Lists MR, CT, DX, but the CT share is not public (TCIA gives no per-modality counts; IDC mirrors only its pathology / derived segmentations): visible once the licence is granted.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>ABIDE II</t>
+          <t>Ivy GAP</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr"/>
@@ -4627,12 +4757,12 @@
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>Pre-op, post-op and follow-up MR</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr">
         <is>
-          <t>Public download</t>
+          <t>Apply</t>
         </is>
       </c>
       <c r="F65" s="8" t="n"/>
@@ -4641,35 +4771,31 @@
       <c r="I65" s="8" t="n"/>
       <c r="J65" s="7" t="inlineStr">
         <is>
-          <t>~1,100 subjects</t>
-        </is>
-      </c>
-      <c r="K65" s="7" t="inlineStr">
-        <is>
-          <t>ASD vs control</t>
-        </is>
-      </c>
+          <t>39 patients, 390 studies, 5,223 series (140 GB)</t>
+        </is>
+      </c>
+      <c r="K65" s="7" t="inlineStr"/>
       <c r="L65" s="7" t="inlineStr"/>
       <c r="M65" s="7" t="inlineStr">
         <is>
-          <t>INDI / FCP (open)</t>
+          <t>TCIA Restricted License; outcomes / genomics in the separate Ivy GAP database (registration)</t>
         </is>
       </c>
       <c r="N65" s="7" t="inlineStr">
         <is>
-          <t>fcon_1000.projects.nitrc.org</t>
+          <t>cancerimagingarchive.net/collection/ivygap</t>
         </is>
       </c>
       <c r="O65" s="7" t="inlineStr">
         <is>
-          <t>BrainDINO's ABIDE count (1,196) exceeds ABIDE I alone.</t>
+          <t>Too small for evaluation; longitudinal / post-op variety only.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>LONG579</t>
+          <t>MU-Glioma-Post</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr"/>
@@ -4680,39 +4806,247 @@
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>T1</t>
+          <t>T1, T1c, T2, FLAIR (post-treatment)</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>Unidentified</t>
+          <t>Candidate</t>
         </is>
       </c>
       <c r="F66" s="8" t="n"/>
       <c r="G66" s="8" t="n"/>
       <c r="H66" s="8" t="n"/>
       <c r="I66" s="8" t="n"/>
-      <c r="J66" s="7" t="inlineStr"/>
+      <c r="J66" s="7" t="inlineStr">
+        <is>
+          <t>~200 patients (unverified)</t>
+        </is>
+      </c>
       <c r="K66" s="7" t="inlineStr">
         <is>
+          <t>Post-treatment segmentation; progression</t>
+        </is>
+      </c>
+      <c r="L66" s="7" t="inlineStr"/>
+      <c r="M66" s="7" t="inlineStr">
+        <is>
+          <t>TCIA (licence to check)</t>
+        </is>
+      </c>
+      <c r="N66" s="7" t="inlineStr">
+        <is>
+          <t>TCIA</t>
+        </is>
+      </c>
+      <c r="O66" s="7" t="inlineStr">
+        <is>
+          <t>Post-treatment glioma with segmentations; candidate response / progression eval.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="7" t="inlineStr">
+        <is>
+          <t>LUMIERE</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr"/>
+      <c r="C67" s="7" t="inlineStr">
+        <is>
+          <t>MRI</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>T1, T1c, T2, FLAIR, longitudinal</t>
+        </is>
+      </c>
+      <c r="E67" s="7" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="F67" s="8" t="n"/>
+      <c r="G67" s="8" t="n"/>
+      <c r="H67" s="8" t="n"/>
+      <c r="I67" s="8" t="n"/>
+      <c r="J67" s="7" t="inlineStr">
+        <is>
+          <t>~90 patients (unverified)</t>
+        </is>
+      </c>
+      <c r="K67" s="7" t="inlineStr">
+        <is>
+          <t>RANO response; progression</t>
+        </is>
+      </c>
+      <c r="L67" s="7" t="inlineStr"/>
+      <c r="M67" s="7" t="inlineStr">
+        <is>
+          <t>Open (licence to check)</t>
+        </is>
+      </c>
+      <c r="N67" s="7" t="inlineStr">
+        <is>
+          <t>figshare (Suter et al. 2022)</t>
+        </is>
+      </c>
+      <c r="O67" s="7" t="inlineStr">
+        <is>
+          <t>Longitudinal glioblastoma with RANO ratings.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>APIS</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr"/>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>CT + MRI</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>Paired NCCT + ADC</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>Candidate</t>
+        </is>
+      </c>
+      <c r="F68" s="8" t="n"/>
+      <c r="G68" s="8" t="n"/>
+      <c r="H68" s="8" t="n"/>
+      <c r="I68" s="8" t="n"/>
+      <c r="J68" s="7" t="inlineStr"/>
+      <c r="K68" s="7" t="inlineStr">
+        <is>
+          <t>Ischemic lesion segmentation (CT and MRI)</t>
+        </is>
+      </c>
+      <c r="L68" s="7" t="inlineStr"/>
+      <c r="M68" s="7" t="inlineStr">
+        <is>
+          <t>Challenge registration</t>
+        </is>
+      </c>
+      <c r="N68" s="7" t="inlineStr">
+        <is>
+          <t>APIS challenge</t>
+        </is>
+      </c>
+      <c r="O68" s="7" t="inlineStr">
+        <is>
+          <t>Paired CT / MRI of the same stroke: a direct modality-agnosticism test.</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>ABIDE II</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr"/>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>MRI</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr">
+        <is>
+          <t>Public download</t>
+        </is>
+      </c>
+      <c r="F69" s="8" t="n"/>
+      <c r="G69" s="8" t="n"/>
+      <c r="H69" s="8" t="n"/>
+      <c r="I69" s="8" t="n"/>
+      <c r="J69" s="7" t="inlineStr">
+        <is>
+          <t>~1,100 subjects</t>
+        </is>
+      </c>
+      <c r="K69" s="7" t="inlineStr">
+        <is>
+          <t>ASD vs control</t>
+        </is>
+      </c>
+      <c r="L69" s="7" t="inlineStr"/>
+      <c r="M69" s="7" t="inlineStr">
+        <is>
+          <t>INDI / FCP (open)</t>
+        </is>
+      </c>
+      <c r="N69" s="7" t="inlineStr">
+        <is>
+          <t>fcon_1000.projects.nitrc.org</t>
+        </is>
+      </c>
+      <c r="O69" s="7" t="inlineStr">
+        <is>
+          <t>BrainDINO's ABIDE count (1,196) exceeds ABIDE I alone.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>LONG579</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr"/>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>MRI</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>T1</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>Unidentified</t>
+        </is>
+      </c>
+      <c r="F70" s="8" t="n"/>
+      <c r="G70" s="8" t="n"/>
+      <c r="H70" s="8" t="n"/>
+      <c r="I70" s="8" t="n"/>
+      <c r="J70" s="7" t="inlineStr"/>
+      <c r="K70" s="7" t="inlineStr">
+        <is>
           <t>Brain age</t>
         </is>
       </c>
-      <c r="L66" s="7" t="inlineStr"/>
-      <c r="M66" s="7" t="inlineStr"/>
-      <c r="N66" s="7" t="inlineStr">
+      <c r="L70" s="7" t="inlineStr"/>
+      <c r="M70" s="7" t="inlineStr"/>
+      <c r="N70" s="7" t="inlineStr">
         <is>
           <t>BrainDINO Supp. Table 2</t>
         </is>
       </c>
-      <c r="O66" s="7" t="inlineStr">
+      <c r="O70" s="7" t="inlineStr">
         <is>
           <t>Part of BrainDINO's brain-age pool; not described in the main text.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O66"/>
+  <autoFilter ref="A1:O70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -4724,7 +5058,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S68"/>
+  <dimension ref="A1:S70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -7852,12 +8186,12 @@
     <row r="50">
       <c r="A50" s="7" t="inlineStr">
         <is>
-          <t>valdo_cmb</t>
+          <t>ucsf_idh</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>VALDO 2021 (small vessel disease)</t>
+          <t>UCSF-PDGM (preoperative diffuse glioma)</t>
         </is>
       </c>
       <c r="C50" s="7" t="inlineStr">
@@ -7867,25 +8201,31 @@
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>segmentation</t>
-        </is>
-      </c>
-      <c r="E50" s="7" t="inlineStr"/>
-      <c r="F50" s="8" t="n"/>
-      <c r="G50" s="8" t="n"/>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>IDH_mutant</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="n">
+        <v>495</v>
+      </c>
+      <c r="G50" s="8" t="n">
+        <v>103</v>
+      </c>
       <c r="H50" s="7" t="inlineStr"/>
-      <c r="I50" s="8" t="n"/>
+      <c r="I50" s="8" t="n">
+        <v>94</v>
+      </c>
       <c r="J50" s="7" t="inlineStr">
         <is>
-          <t>Suite only</t>
+          <t>Suite only: not selected</t>
         </is>
       </c>
       <c r="K50" s="7" t="inlineStr"/>
-      <c r="L50" s="7" t="inlineStr">
-        <is>
-          <t>Dice</t>
-        </is>
-      </c>
+      <c r="L50" s="7" t="inlineStr"/>
       <c r="M50" s="9" t="n"/>
       <c r="N50" s="9" t="n"/>
       <c r="O50" s="9" t="n"/>
@@ -7894,19 +8234,19 @@
       <c r="R50" s="7" t="inlineStr"/>
       <c r="S50" s="7" t="inlineStr">
         <is>
-          <t>Cerebral microbleeds.</t>
+          <t>Added 2026-10-28; not yet in the benchmark. Seen-target for runs that train glioma_idh (TCGA).</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="7" t="inlineStr">
         <is>
-          <t>valdo_lacunes</t>
+          <t>ucsf_lgg</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>VALDO 2021 (small vessel disease)</t>
+          <t>UCSF-PDGM (preoperative diffuse glioma)</t>
         </is>
       </c>
       <c r="C51" s="7" t="inlineStr">
@@ -7916,25 +8256,31 @@
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>segmentation</t>
-        </is>
-      </c>
-      <c r="E51" s="7" t="inlineStr"/>
-      <c r="F51" s="8" t="n"/>
-      <c r="G51" s="8" t="n"/>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>grade_2_3</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="n">
+        <v>495</v>
+      </c>
+      <c r="G51" s="8" t="n">
+        <v>99</v>
+      </c>
       <c r="H51" s="7" t="inlineStr"/>
-      <c r="I51" s="8" t="n"/>
+      <c r="I51" s="8" t="n">
+        <v>94</v>
+      </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
-          <t>Suite only</t>
+          <t>Suite only: not selected</t>
         </is>
       </c>
       <c r="K51" s="7" t="inlineStr"/>
-      <c r="L51" s="7" t="inlineStr">
-        <is>
-          <t>Dice</t>
-        </is>
-      </c>
+      <c r="L51" s="7" t="inlineStr"/>
       <c r="M51" s="9" t="n"/>
       <c r="N51" s="9" t="n"/>
       <c r="O51" s="9" t="n"/>
@@ -7943,39 +8289,49 @@
       <c r="R51" s="7" t="inlineStr"/>
       <c r="S51" s="7" t="inlineStr">
         <is>
-          <t>Lacunes.</t>
+          <t>Added 2026-10-28; WHO grade &lt; 4. Seen-target for runs that train glioma_lower_grade.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="7" t="inlineStr">
         <is>
-          <t>center_tbi_lesions</t>
+          <t>ucsf_mgmt</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>CENTER-TBI</t>
+          <t>UCSF-PDGM (preoperative diffuse glioma)</t>
         </is>
       </c>
       <c r="C52" s="7" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>MRI</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>multi-label</t>
-        </is>
-      </c>
-      <c r="E52" s="7" t="inlineStr"/>
-      <c r="F52" s="8" t="n"/>
-      <c r="G52" s="8" t="n"/>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>MGMT_methylated</t>
+        </is>
+      </c>
+      <c r="F52" s="8" t="n">
+        <v>351</v>
+      </c>
+      <c r="G52" s="8" t="n">
+        <v>247</v>
+      </c>
       <c r="H52" s="7" t="inlineStr"/>
-      <c r="I52" s="8" t="n"/>
+      <c r="I52" s="8" t="n">
+        <v>67</v>
+      </c>
       <c r="J52" s="7" t="inlineStr">
         <is>
-          <t>Planned: needs data</t>
+          <t>Suite only: not selected</t>
         </is>
       </c>
       <c r="K52" s="7" t="inlineStr"/>
@@ -7986,22 +8342,26 @@
       <c r="P52" s="7" t="inlineStr"/>
       <c r="Q52" s="9" t="n"/>
       <c r="R52" s="7" t="inlineStr"/>
-      <c r="S52" s="7" t="inlineStr"/>
+      <c r="S52" s="7" t="inlineStr">
+        <is>
+          <t>Added 2026-10-28; IDH-wildtype glioblastoma only.</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="7" t="inlineStr">
         <is>
-          <t>sinoct_triage</t>
+          <t>ucsf_survival_12m</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>SinoCT</t>
+          <t>UCSF-PDGM (preoperative diffuse glioma)</t>
         </is>
       </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
-          <t>CT</t>
+          <t>MRI</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
@@ -8009,14 +8369,24 @@
           <t>binary</t>
         </is>
       </c>
-      <c r="E53" s="7" t="inlineStr"/>
-      <c r="F53" s="8" t="n"/>
-      <c r="G53" s="8" t="n"/>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>survived_12m</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="n">
+        <v>395</v>
+      </c>
+      <c r="G53" s="8" t="n">
+        <v>278</v>
+      </c>
       <c r="H53" s="7" t="inlineStr"/>
-      <c r="I53" s="8" t="n"/>
+      <c r="I53" s="8" t="n">
+        <v>77</v>
+      </c>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>Planned: needs data</t>
+          <t>Suite only: not selected</t>
         </is>
       </c>
       <c r="K53" s="7" t="inlineStr"/>
@@ -8026,22 +8396,22 @@
       <c r="O53" s="9" t="n"/>
       <c r="P53" s="7" t="inlineStr"/>
       <c r="Q53" s="9" t="n"/>
-      <c r="R53" s="7" t="inlineStr">
-        <is>
-          <t>CT-FM</t>
-        </is>
-      </c>
-      <c r="S53" s="7" t="inlineStr"/>
+      <c r="R53" s="7" t="inlineStr"/>
+      <c r="S53" s="7" t="inlineStr">
+        <is>
+          <t>Added 2026-10-28; alive with &lt; 1 y follow-up dropped. Seen-target for glioma_survival_12m runs.</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="7" t="inlineStr">
         <is>
-          <t>adni_3class</t>
+          <t>valdo_cmb</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>ADNI</t>
+          <t>VALDO 2021 (small vessel disease)</t>
         </is>
       </c>
       <c r="C54" s="7" t="inlineStr">
@@ -8051,7 +8421,7 @@
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>multiclass</t>
+          <t>segmentation</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr"/>
@@ -8061,32 +8431,36 @@
       <c r="I54" s="8" t="n"/>
       <c r="J54" s="7" t="inlineStr">
         <is>
-          <t>Planned: needs data</t>
+          <t>Suite only</t>
         </is>
       </c>
       <c r="K54" s="7" t="inlineStr"/>
-      <c r="L54" s="7" t="inlineStr"/>
+      <c r="L54" s="7" t="inlineStr">
+        <is>
+          <t>Dice</t>
+        </is>
+      </c>
       <c r="M54" s="9" t="n"/>
       <c r="N54" s="9" t="n"/>
       <c r="O54" s="9" t="n"/>
       <c r="P54" s="7" t="inlineStr"/>
       <c r="Q54" s="9" t="n"/>
-      <c r="R54" s="7" t="inlineStr">
-        <is>
-          <t>BrainDINO</t>
-        </is>
-      </c>
-      <c r="S54" s="7" t="inlineStr"/>
+      <c r="R54" s="7" t="inlineStr"/>
+      <c r="S54" s="7" t="inlineStr">
+        <is>
+          <t>Cerebral microbleeds.</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="7" t="inlineStr">
         <is>
-          <t>adni_cn_ad</t>
+          <t>valdo_lacunes</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>ADNI</t>
+          <t>VALDO 2021 (small vessel disease)</t>
         </is>
       </c>
       <c r="C55" s="7" t="inlineStr">
@@ -8096,7 +8470,7 @@
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>binary</t>
+          <t>segmentation</t>
         </is>
       </c>
       <c r="E55" s="7" t="inlineStr"/>
@@ -8106,42 +8480,46 @@
       <c r="I55" s="8" t="n"/>
       <c r="J55" s="7" t="inlineStr">
         <is>
-          <t>Planned: needs data</t>
+          <t>Suite only</t>
         </is>
       </c>
       <c r="K55" s="7" t="inlineStr"/>
-      <c r="L55" s="7" t="inlineStr"/>
+      <c r="L55" s="7" t="inlineStr">
+        <is>
+          <t>Dice</t>
+        </is>
+      </c>
       <c r="M55" s="9" t="n"/>
       <c r="N55" s="9" t="n"/>
       <c r="O55" s="9" t="n"/>
       <c r="P55" s="7" t="inlineStr"/>
       <c r="Q55" s="9" t="n"/>
-      <c r="R55" s="7" t="inlineStr">
-        <is>
-          <t>BrainDINO; BrainNorm; NeuroVFM</t>
-        </is>
-      </c>
-      <c r="S55" s="7" t="inlineStr"/>
+      <c r="R55" s="7" t="inlineStr"/>
+      <c r="S55" s="7" t="inlineStr">
+        <is>
+          <t>Lacunes.</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="7" t="inlineStr">
         <is>
-          <t>adni_cn_mci</t>
+          <t>center_tbi_lesions</t>
         </is>
       </c>
       <c r="B56" s="7" t="inlineStr">
         <is>
-          <t>ADNI</t>
+          <t>CENTER-TBI</t>
         </is>
       </c>
       <c r="C56" s="7" t="inlineStr">
         <is>
-          <t>MRI</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
         <is>
-          <t>binary</t>
+          <t>multi-label</t>
         </is>
       </c>
       <c r="E56" s="7" t="inlineStr"/>
@@ -8161,32 +8539,28 @@
       <c r="O56" s="9" t="n"/>
       <c r="P56" s="7" t="inlineStr"/>
       <c r="Q56" s="9" t="n"/>
-      <c r="R56" s="7" t="inlineStr">
-        <is>
-          <t>BrainDINO</t>
-        </is>
-      </c>
+      <c r="R56" s="7" t="inlineStr"/>
       <c r="S56" s="7" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="7" t="inlineStr">
         <is>
-          <t>adni_mmse</t>
+          <t>sinoct_triage</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>ADNI</t>
+          <t>SinoCT</t>
         </is>
       </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
-          <t>MRI</t>
+          <t>CT</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>regression</t>
+          <t>binary</t>
         </is>
       </c>
       <c r="E57" s="7" t="inlineStr"/>
@@ -8206,13 +8580,17 @@
       <c r="O57" s="9" t="n"/>
       <c r="P57" s="7" t="inlineStr"/>
       <c r="Q57" s="9" t="n"/>
-      <c r="R57" s="7" t="inlineStr"/>
+      <c r="R57" s="7" t="inlineStr">
+        <is>
+          <t>CT-FM</t>
+        </is>
+      </c>
       <c r="S57" s="7" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="7" t="inlineStr">
         <is>
-          <t>adni_smci_pmci</t>
+          <t>adni_3class</t>
         </is>
       </c>
       <c r="B58" s="7" t="inlineStr">
@@ -8227,7 +8605,7 @@
       </c>
       <c r="D58" s="7" t="inlineStr">
         <is>
-          <t>binary</t>
+          <t>multiclass</t>
         </is>
       </c>
       <c r="E58" s="7" t="inlineStr"/>
@@ -8249,7 +8627,7 @@
       <c r="Q58" s="9" t="n"/>
       <c r="R58" s="7" t="inlineStr">
         <is>
-          <t>BrainNorm; classic ML literature</t>
+          <t>BrainDINO</t>
         </is>
       </c>
       <c r="S58" s="7" t="inlineStr"/>
@@ -8257,12 +8635,12 @@
     <row r="59">
       <c r="A59" s="7" t="inlineStr">
         <is>
-          <t>aibl_cn_ad</t>
+          <t>adni_cn_ad</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>AIBL</t>
+          <t>ADNI</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
@@ -8292,28 +8670,32 @@
       <c r="O59" s="9" t="n"/>
       <c r="P59" s="7" t="inlineStr"/>
       <c r="Q59" s="9" t="n"/>
-      <c r="R59" s="7" t="inlineStr"/>
+      <c r="R59" s="7" t="inlineStr">
+        <is>
+          <t>BrainDINO; BrainNorm; NeuroVFM</t>
+        </is>
+      </c>
       <c r="S59" s="7" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="7" t="inlineStr">
         <is>
-          <t>apis_seg</t>
+          <t>adni_cn_mci</t>
         </is>
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>APIS</t>
+          <t>ADNI</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
         <is>
-          <t>CT + MRI</t>
+          <t>MRI</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
         <is>
-          <t>segmentation</t>
+          <t>binary</t>
         </is>
       </c>
       <c r="E60" s="7" t="inlineStr"/>
@@ -8333,18 +8715,22 @@
       <c r="O60" s="9" t="n"/>
       <c r="P60" s="7" t="inlineStr"/>
       <c r="Q60" s="9" t="n"/>
-      <c r="R60" s="7" t="inlineStr"/>
+      <c r="R60" s="7" t="inlineStr">
+        <is>
+          <t>BrainDINO</t>
+        </is>
+      </c>
       <c r="S60" s="7" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="7" t="inlineStr">
         <is>
-          <t>brats_mets</t>
+          <t>adni_mmse</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>BraTS 2023-METS</t>
+          <t>ADNI</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
@@ -8354,7 +8740,7 @@
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>segmentation</t>
+          <t>regression</t>
         </is>
       </c>
       <c r="E61" s="7" t="inlineStr"/>
@@ -8374,32 +8760,28 @@
       <c r="O61" s="9" t="n"/>
       <c r="P61" s="7" t="inlineStr"/>
       <c r="Q61" s="9" t="n"/>
-      <c r="R61" s="7" t="inlineStr">
-        <is>
-          <t>BrainDINO</t>
-        </is>
-      </c>
+      <c r="R61" s="7" t="inlineStr"/>
       <c r="S61" s="7" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="7" t="inlineStr">
         <is>
-          <t>oasis3_cdr</t>
+          <t>adni_smci_pmci</t>
         </is>
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>OASIS-3</t>
+          <t>ADNI</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
         <is>
-          <t>CT + MRI</t>
+          <t>MRI</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
         <is>
-          <t>binary / ordinal</t>
+          <t>binary</t>
         </is>
       </c>
       <c r="E62" s="7" t="inlineStr"/>
@@ -8419,18 +8801,22 @@
       <c r="O62" s="9" t="n"/>
       <c r="P62" s="7" t="inlineStr"/>
       <c r="Q62" s="9" t="n"/>
-      <c r="R62" s="7" t="inlineStr"/>
+      <c r="R62" s="7" t="inlineStr">
+        <is>
+          <t>BrainNorm; classic ML literature</t>
+        </is>
+      </c>
       <c r="S62" s="7" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="7" t="inlineStr">
         <is>
-          <t>ppmi_pd</t>
+          <t>aibl_cn_ad</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>PPMI</t>
+          <t>AIBL</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
@@ -8460,22 +8846,18 @@
       <c r="O63" s="9" t="n"/>
       <c r="P63" s="7" t="inlineStr"/>
       <c r="Q63" s="9" t="n"/>
-      <c r="R63" s="7" t="inlineStr">
-        <is>
-          <t>BrainDINO</t>
-        </is>
-      </c>
+      <c r="R63" s="7" t="inlineStr"/>
       <c r="S63" s="7" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="7" t="inlineStr">
         <is>
-          <t>rsna_ica_aneurysm</t>
+          <t>apis_seg</t>
         </is>
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>RSNA Intracranial Aneurysm</t>
+          <t>APIS</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
@@ -8485,7 +8867,7 @@
       </c>
       <c r="D64" s="7" t="inlineStr">
         <is>
-          <t>binary + location</t>
+          <t>segmentation</t>
         </is>
       </c>
       <c r="E64" s="7" t="inlineStr"/>
@@ -8505,22 +8887,18 @@
       <c r="O64" s="9" t="n"/>
       <c r="P64" s="7" t="inlineStr"/>
       <c r="Q64" s="9" t="n"/>
-      <c r="R64" s="7" t="inlineStr">
-        <is>
-          <t>RSNA 2025 Kaggle</t>
-        </is>
-      </c>
+      <c r="R64" s="7" t="inlineStr"/>
       <c r="S64" s="7" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="7" t="inlineStr">
         <is>
-          <t>ucsf_pdgm_grade</t>
+          <t>brats_mets</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>UCSF-PDGM</t>
+          <t>BraTS 2023-METS</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
@@ -8530,7 +8908,7 @@
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>binary</t>
+          <t>segmentation</t>
         </is>
       </c>
       <c r="E65" s="7" t="inlineStr"/>
@@ -8550,28 +8928,32 @@
       <c r="O65" s="9" t="n"/>
       <c r="P65" s="7" t="inlineStr"/>
       <c r="Q65" s="9" t="n"/>
-      <c r="R65" s="7" t="inlineStr"/>
+      <c r="R65" s="7" t="inlineStr">
+        <is>
+          <t>BrainDINO</t>
+        </is>
+      </c>
       <c r="S65" s="7" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="7" t="inlineStr">
         <is>
-          <t>ucsf_pdgm_idh</t>
+          <t>oasis3_cdr</t>
         </is>
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>UCSF-PDGM</t>
+          <t>OASIS-3</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
         <is>
-          <t>MRI</t>
+          <t>CT + MRI</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
         <is>
-          <t>binary</t>
+          <t>binary / ordinal</t>
         </is>
       </c>
       <c r="E66" s="7" t="inlineStr"/>
@@ -8591,22 +8973,18 @@
       <c r="O66" s="9" t="n"/>
       <c r="P66" s="7" t="inlineStr"/>
       <c r="Q66" s="9" t="n"/>
-      <c r="R66" s="7" t="inlineStr">
-        <is>
-          <t>BrainDINO</t>
-        </is>
-      </c>
+      <c r="R66" s="7" t="inlineStr"/>
       <c r="S66" s="7" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="7" t="inlineStr">
         <is>
-          <t>upenn_gbm_os</t>
+          <t>ppmi_pd</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>UPENN-GBM</t>
+          <t>PPMI</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
@@ -8616,7 +8994,7 @@
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>survival (C-index)</t>
+          <t>binary</t>
         </is>
       </c>
       <c r="E67" s="7" t="inlineStr"/>
@@ -8646,22 +9024,22 @@
     <row r="68">
       <c r="A68" s="7" t="inlineStr">
         <is>
-          <t>upenn_gbm_os_1y</t>
+          <t>rsna_ica_aneurysm</t>
         </is>
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>UPENN-GBM</t>
+          <t>RSNA Intracranial Aneurysm</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
         <is>
-          <t>MRI</t>
+          <t>CT + MRI</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
         <is>
-          <t>binary</t>
+          <t>binary + location</t>
         </is>
       </c>
       <c r="E68" s="7" t="inlineStr"/>
@@ -8683,13 +9061,103 @@
       <c r="Q68" s="9" t="n"/>
       <c r="R68" s="7" t="inlineStr">
         <is>
+          <t>RSNA 2025 Kaggle</t>
+        </is>
+      </c>
+      <c r="S68" s="7" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="7" t="inlineStr">
+        <is>
+          <t>upenn_gbm_os</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>UPENN-GBM</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>MRI</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>survival (C-index)</t>
+        </is>
+      </c>
+      <c r="E69" s="7" t="inlineStr"/>
+      <c r="F69" s="8" t="n"/>
+      <c r="G69" s="8" t="n"/>
+      <c r="H69" s="7" t="inlineStr"/>
+      <c r="I69" s="8" t="n"/>
+      <c r="J69" s="7" t="inlineStr">
+        <is>
+          <t>Planned: needs data</t>
+        </is>
+      </c>
+      <c r="K69" s="7" t="inlineStr"/>
+      <c r="L69" s="7" t="inlineStr"/>
+      <c r="M69" s="9" t="n"/>
+      <c r="N69" s="9" t="n"/>
+      <c r="O69" s="9" t="n"/>
+      <c r="P69" s="7" t="inlineStr"/>
+      <c r="Q69" s="9" t="n"/>
+      <c r="R69" s="7" t="inlineStr">
+        <is>
           <t>BrainDINO</t>
         </is>
       </c>
-      <c r="S68" s="7" t="inlineStr"/>
+      <c r="S69" s="7" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>upenn_gbm_os_1y</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>UPENN-GBM</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>MRI</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>binary</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr"/>
+      <c r="F70" s="8" t="n"/>
+      <c r="G70" s="8" t="n"/>
+      <c r="H70" s="7" t="inlineStr"/>
+      <c r="I70" s="8" t="n"/>
+      <c r="J70" s="7" t="inlineStr">
+        <is>
+          <t>Planned: needs data</t>
+        </is>
+      </c>
+      <c r="K70" s="7" t="inlineStr"/>
+      <c r="L70" s="7" t="inlineStr"/>
+      <c r="M70" s="9" t="n"/>
+      <c r="N70" s="9" t="n"/>
+      <c r="O70" s="9" t="n"/>
+      <c r="P70" s="7" t="inlineStr"/>
+      <c r="Q70" s="9" t="n"/>
+      <c r="R70" s="7" t="inlineStr">
+        <is>
+          <t>BrainDINO</t>
+        </is>
+      </c>
+      <c r="S70" s="7" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S68"/>
+  <autoFilter ref="A1:S70"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
@@ -8775,7 +9243,7 @@
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (25,058), Healthy Brain Network (FOMO) (5,383), NKI-Rockland (FOMO) (3,413), CoRR (FOMO) (2,001), Infant MRI (FOMO) (1,249), SLIM longitudinal (FOMO) (759), WAND (FOMO) (597), BrainLat (FOMO) (413), FOMO cohort: nigerian (203), Cuban Human Brain Mapping (FOMO) (153), FOMO cohort: hbnssi (137), FOMO cohort: wayne (134), FOMO cohort: abd (131), ACPI (FOMO) (122), FOMO cohort: ageility (98), FOMO cohort: yale_highres (93), FOMO cohort: cunmet (45), Tao Wu Parkinson's (FOMO) (30), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (25,058), Healthy Brain Network (FOMO) (5,383), NKI-Rockland (FOMO) (3,413), CoRR (FOMO) (2,001), Infant MRI (FOMO) (1,249), SLIM longitudinal (FOMO) (759), WAND (FOMO) (597), BrainLat (FOMO) (413), fomo_nigerian (203), Cuban Human Brain Mapping (FOMO) (153), fomo_hbnssi (137), fomo_wayne (134), fomo_abd (131), ACPI (FOMO) (122), fomo_ageility (98), fomo_yale_highres (93), fomo_cunmet (45), Tao Wu Parkinson's (FOMO) (30), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F2" s="8" t="n">
@@ -8809,7 +9277,7 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (24,037), RSNA Intracranial Hemorrhage 2019 (12,384), BraTS glioma (2021 / 2023 / 2024 GLI) (6,233), Healthy Brain Network (FOMO) (4,797), NKI-Rockland (FOMO) (4,364), BraTS-MEN 2023 (2,749), CoRR (FOMO) (2,002), BraTS-GoAT 2024 (1,108), IXI (869), ABIDE I (819), SLIM longitudinal (FOMO) (700), AOMIC ID1000 (696), WAND (FOMO) (492), BrainLat (FOMO) (452), M4Raw low-field (FOMO) (442), FOMO cohort: wayne (424), BraTS-PED 2023 (408), OASIS-1 (314), HemSeg-500 (280), FOMO cohort: yale_highres (195), FOMO cohort: nigerian (176), OASIS-2 (longitudinal) (176), AOMIC PIOP2 (169), AOMIC PIOP1 (162), FOMO cohort: abd (124), Pixar (OpenNeuro ds000228) (115), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: hbnssi (87), BHSD (brain hemorrhage segmentation) (84), Infant MRI (FOMO) (68), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (24,037), RSNA Intracranial Hemorrhage 2019 (12,384), BraTS glioma (2021 / 2023 / 2024 GLI) (6,233), Healthy Brain Network (FOMO) (4,797), NKI-Rockland (FOMO) (4,364), BraTS-MEN 2023 (2,749), CoRR (FOMO) (2,002), BraTS-GoAT 2024 (1,108), IXI (869), ABIDE I (819), SLIM longitudinal (FOMO) (700), AOMIC ID1000 (696), WAND (FOMO) (492), BrainLat (FOMO) (452), M4Raw low-field (FOMO) (442), fomo_wayne (424), BraTS-PED 2023 (408), OASIS-1 (314), HemSeg-500 (280), fomo_yale_highres (195), fomo_nigerian (176), OASIS-2 (longitudinal) (176), AOMIC PIOP2 (169), AOMIC PIOP1 (162), fomo_abd (124), Pixar (OpenNeuro ds000228) (115), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), ACPI (FOMO) (98), fomo_ageility (98), fomo_hbnssi (87), BHSD (brain hemorrhage segmentation) (84), Infant MRI (FOMO) (68), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F3" s="8" t="n">
@@ -8843,7 +9311,7 @@
       </c>
       <c r="E4" s="7" t="inlineStr">
         <is>
-          <t>RSNA Intracranial Hemorrhage 2019 (17,679), Healthy Brain Network (FOMO) (5,108), NKI-Rockland (FOMO) (4,425), CoRR (FOMO) (2,008), IXI (869), ABIDE I (823), SLIM longitudinal (FOMO) (769), AOMIC ID1000 (696), WAND (FOMO) (529), M4Raw low-field (FOMO) (468), BrainLat (FOMO) (455), FOMO cohort: wayne (444), Infant MRI (FOMO) (428), HemSeg-500 (382), OASIS-1 (315), FOMO cohort: yale_highres (196), FOMO cohort: nigerian (195), OASIS-2 (longitudinal) (176), AOMIC PIOP2 (169), AOMIC PIOP1 (162), Cuban Human Brain Mapping (FOMO) (142), FOMO cohort: beijing (134), BHSD (brain hemorrhage segmentation) (132), FOMO cohort: hbnssi (126), FOMO cohort: abd (125), Pixar (OpenNeuro ds000228) (115), ACPI (FOMO) (102), FOMO cohort: ageility (98), AHEAD 7T (FOMO) (79), FOMO cohort: cunmet (38), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), FOMO cohort: cleveland (23)</t>
+          <t>RSNA Intracranial Hemorrhage 2019 (17,679), Healthy Brain Network (FOMO) (5,108), NKI-Rockland (FOMO) (4,425), CoRR (FOMO) (2,008), IXI (869), ABIDE I (823), SLIM longitudinal (FOMO) (769), AOMIC ID1000 (696), WAND (FOMO) (529), M4Raw low-field (FOMO) (468), BrainLat (FOMO) (455), fomo_wayne (444), Infant MRI (FOMO) (428), HemSeg-500 (382), OASIS-1 (315), fomo_yale_highres (196), fomo_nigerian (195), OASIS-2 (longitudinal) (176), AOMIC PIOP2 (169), AOMIC PIOP1 (162), Cuban Human Brain Mapping (FOMO) (142), fomo_beijing (134), BHSD (brain hemorrhage segmentation) (132), fomo_hbnssi (126), fomo_abd (125), Pixar (OpenNeuro ds000228) (115), ACPI (FOMO) (102), fomo_ageility (98), AHEAD 7T (FOMO) (79), fomo_cunmet (38), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F4" s="8" t="n">
@@ -8877,7 +9345,7 @@
       </c>
       <c r="E5" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (24,037), RSNA Intracranial Hemorrhage 2019 (12,384), BraTS glioma (2021 / 2023 / 2024 GLI) (6,233), Healthy Brain Network (FOMO) (4,797), NKI-Rockland (FOMO) (4,364), BraTS-MEN 2023 (2,749), CoRR (FOMO) (2,002), BraTS-GoAT 2024 (1,108), IXI (869), ABIDE I (819), SLIM longitudinal (FOMO) (700), AOMIC ID1000 (696), WAND (FOMO) (492), BrainLat (FOMO) (452), M4Raw low-field (FOMO) (442), FOMO cohort: wayne (424), BraTS-PED 2023 (408), OASIS-1 (314), HemSeg-500 (280), FOMO cohort: yale_highres (195), FOMO cohort: nigerian (176), OASIS-2 (longitudinal) (176), AOMIC PIOP2 (169), AOMIC PIOP1 (162), FOMO cohort: abd (124), Pixar (OpenNeuro ds000228) (115), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: hbnssi (87), BHSD (brain hemorrhage segmentation) (84), Infant MRI (FOMO) (68), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (24,037), RSNA Intracranial Hemorrhage 2019 (12,384), BraTS glioma (2021 / 2023 / 2024 GLI) (6,233), Healthy Brain Network (FOMO) (4,797), NKI-Rockland (FOMO) (4,364), BraTS-MEN 2023 (2,749), CoRR (FOMO) (2,002), BraTS-GoAT 2024 (1,108), IXI (869), ABIDE I (819), SLIM longitudinal (FOMO) (700), AOMIC ID1000 (696), WAND (FOMO) (492), BrainLat (FOMO) (452), M4Raw low-field (FOMO) (442), fomo_wayne (424), BraTS-PED 2023 (408), OASIS-1 (314), HemSeg-500 (280), fomo_yale_highres (195), fomo_nigerian (176), OASIS-2 (longitudinal) (176), AOMIC PIOP2 (169), AOMIC PIOP1 (162), fomo_abd (124), Pixar (OpenNeuro ds000228) (115), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), ACPI (FOMO) (98), fomo_ageility (98), fomo_hbnssi (87), BHSD (brain hemorrhage segmentation) (84), Infant MRI (FOMO) (68), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F5" s="8" t="n">
@@ -8914,7 +9382,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="8" t="n">
-        <v>515</v>
+        <v>467</v>
       </c>
       <c r="H6" s="7" t="inlineStr">
         <is>
@@ -8944,7 +9412,7 @@
         <v>0</v>
       </c>
       <c r="G7" s="8" t="n">
-        <v>515</v>
+        <v>467</v>
       </c>
       <c r="H7" s="7" t="inlineStr">
         <is>
@@ -8974,7 +9442,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="8" t="n">
-        <v>515</v>
+        <v>467</v>
       </c>
       <c r="H8" s="7" t="inlineStr">
         <is>
@@ -9004,7 +9472,7 @@
         <v>0</v>
       </c>
       <c r="G9" s="8" t="n">
-        <v>515</v>
+        <v>467</v>
       </c>
       <c r="H9" s="7" t="inlineStr">
         <is>
@@ -9034,7 +9502,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="8" t="n">
-        <v>515</v>
+        <v>467</v>
       </c>
       <c r="H10" s="7" t="inlineStr">
         <is>
@@ -9064,7 +9532,7 @@
         <v>0</v>
       </c>
       <c r="G11" s="8" t="n">
-        <v>515</v>
+        <v>467</v>
       </c>
       <c r="H11" s="7" t="inlineStr">
         <is>
@@ -9495,7 +9963,7 @@
       </c>
       <c r="E24" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (24,037), RSNA Intracranial Hemorrhage 2019 (12,384), BraTS glioma (2021 / 2023 / 2024 GLI) (6,233), Healthy Brain Network (FOMO) (4,797), NKI-Rockland (FOMO) (4,364), BraTS-MEN 2023 (2,749), CoRR (FOMO) (2,002), BraTS-GoAT 2024 (1,108), IXI (869), ABIDE I (819), SLIM longitudinal (FOMO) (700), AOMIC ID1000 (696), WAND (FOMO) (492), BrainLat (FOMO) (452), M4Raw low-field (FOMO) (442), FOMO cohort: wayne (424), BraTS-PED 2023 (408), OASIS-1 (314), HemSeg-500 (280), FOMO cohort: yale_highres (195), FOMO cohort: nigerian (176), OASIS-2 (longitudinal) (176), AOMIC PIOP2 (169), AOMIC PIOP1 (162), FOMO cohort: abd (124), Pixar (OpenNeuro ds000228) (115), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: hbnssi (87), BHSD (brain hemorrhage segmentation) (84), Infant MRI (FOMO) (68), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (24,037), RSNA Intracranial Hemorrhage 2019 (12,384), BraTS glioma (2021 / 2023 / 2024 GLI) (6,233), Healthy Brain Network (FOMO) (4,797), NKI-Rockland (FOMO) (4,364), BraTS-MEN 2023 (2,749), CoRR (FOMO) (2,002), BraTS-GoAT 2024 (1,108), IXI (869), ABIDE I (819), SLIM longitudinal (FOMO) (700), AOMIC ID1000 (696), WAND (FOMO) (492), BrainLat (FOMO) (452), M4Raw low-field (FOMO) (442), fomo_wayne (424), BraTS-PED 2023 (408), OASIS-1 (314), HemSeg-500 (280), fomo_yale_highres (195), fomo_nigerian (176), OASIS-2 (longitudinal) (176), AOMIC PIOP2 (169), AOMIC PIOP1 (162), fomo_abd (124), Pixar (OpenNeuro ds000228) (115), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), ACPI (FOMO) (98), fomo_ageility (98), fomo_hbnssi (87), BHSD (brain hemorrhage segmentation) (84), Infant MRI (FOMO) (68), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F24" s="8" t="n">
@@ -9627,7 +10095,7 @@
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), FOMO cohort: wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), FOMO cohort: yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), FOMO cohort: nigerian (139), OASIS-2 (longitudinal) (138), FOMO cohort: hbnssi (137), FOMO cohort: beijing (135), FOMO cohort: abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), FOMO cohort: ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), FOMO cohort: cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), fomo_wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), fomo_yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), fomo_nigerian (139), OASIS-2 (longitudinal) (138), fomo_hbnssi (137), fomo_beijing (135), fomo_abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), fomo_ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), fomo_cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F28" s="8" t="n">
@@ -9661,7 +10129,7 @@
       </c>
       <c r="E29" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), FOMO cohort: wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), FOMO cohort: yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), FOMO cohort: nigerian (139), OASIS-2 (longitudinal) (138), FOMO cohort: hbnssi (137), FOMO cohort: beijing (135), FOMO cohort: abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), FOMO cohort: ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), FOMO cohort: cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), fomo_wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), fomo_yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), fomo_nigerian (139), OASIS-2 (longitudinal) (138), fomo_hbnssi (137), fomo_beijing (135), fomo_abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), fomo_ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), fomo_cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F29" s="8" t="n">
@@ -9695,7 +10163,7 @@
       </c>
       <c r="E30" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), FOMO cohort: wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), FOMO cohort: yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), FOMO cohort: nigerian (139), OASIS-2 (longitudinal) (138), FOMO cohort: hbnssi (137), FOMO cohort: beijing (135), FOMO cohort: abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), FOMO cohort: ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), FOMO cohort: cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), fomo_wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), fomo_yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), fomo_nigerian (139), OASIS-2 (longitudinal) (138), fomo_hbnssi (137), fomo_beijing (135), fomo_abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), fomo_ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), fomo_cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F30" s="8" t="n">
@@ -9729,7 +10197,7 @@
       </c>
       <c r="E31" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), FOMO cohort: wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), FOMO cohort: yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), FOMO cohort: nigerian (139), OASIS-2 (longitudinal) (138), FOMO cohort: hbnssi (137), FOMO cohort: beijing (135), FOMO cohort: abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), FOMO cohort: ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), FOMO cohort: cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), fomo_wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), fomo_yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), fomo_nigerian (139), OASIS-2 (longitudinal) (138), fomo_hbnssi (137), fomo_beijing (135), fomo_abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), fomo_ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), fomo_cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F31" s="8" t="n">
@@ -9763,7 +10231,7 @@
       </c>
       <c r="E32" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), FOMO cohort: wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), FOMO cohort: yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), FOMO cohort: nigerian (139), OASIS-2 (longitudinal) (138), FOMO cohort: hbnssi (137), FOMO cohort: beijing (135), FOMO cohort: abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), FOMO cohort: ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), FOMO cohort: cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), fomo_wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), fomo_yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), fomo_nigerian (139), OASIS-2 (longitudinal) (138), fomo_hbnssi (137), fomo_beijing (135), fomo_abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), fomo_ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), fomo_cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F32" s="8" t="n">
@@ -9797,7 +10265,7 @@
       </c>
       <c r="E33" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), FOMO cohort: wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), FOMO cohort: yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), FOMO cohort: nigerian (139), OASIS-2 (longitudinal) (138), FOMO cohort: hbnssi (137), FOMO cohort: beijing (135), FOMO cohort: abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), FOMO cohort: ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), FOMO cohort: cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), fomo_wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), fomo_yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), fomo_nigerian (139), OASIS-2 (longitudinal) (138), fomo_hbnssi (137), fomo_beijing (135), fomo_abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), fomo_ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), fomo_cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F33" s="8" t="n">
@@ -9831,7 +10299,7 @@
       </c>
       <c r="E34" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), FOMO cohort: wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), FOMO cohort: yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), FOMO cohort: nigerian (139), OASIS-2 (longitudinal) (138), FOMO cohort: hbnssi (137), FOMO cohort: beijing (135), FOMO cohort: abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), FOMO cohort: ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), FOMO cohort: cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), fomo_wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), fomo_yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), fomo_nigerian (139), OASIS-2 (longitudinal) (138), fomo_hbnssi (137), fomo_beijing (135), fomo_abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), fomo_ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), fomo_cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F34" s="8" t="n">
@@ -9865,7 +10333,7 @@
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), FOMO cohort: wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), FOMO cohort: yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), FOMO cohort: nigerian (139), OASIS-2 (longitudinal) (138), FOMO cohort: hbnssi (137), FOMO cohort: beijing (135), FOMO cohort: abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), FOMO cohort: ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), FOMO cohort: cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), fomo_wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), fomo_yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), fomo_nigerian (139), OASIS-2 (longitudinal) (138), fomo_hbnssi (137), fomo_beijing (135), fomo_abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), fomo_ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), fomo_cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F35" s="8" t="n">
@@ -9899,7 +10367,7 @@
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), FOMO cohort: wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), FOMO cohort: yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), FOMO cohort: nigerian (139), OASIS-2 (longitudinal) (138), FOMO cohort: hbnssi (137), FOMO cohort: beijing (135), FOMO cohort: abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), FOMO cohort: ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), FOMO cohort: cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), fomo_wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), fomo_yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), fomo_nigerian (139), OASIS-2 (longitudinal) (138), fomo_hbnssi (137), fomo_beijing (135), fomo_abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), fomo_ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), fomo_cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F36" s="8" t="n">
@@ -9933,7 +10401,7 @@
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), FOMO cohort: wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), FOMO cohort: yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), FOMO cohort: nigerian (139), OASIS-2 (longitudinal) (138), FOMO cohort: hbnssi (137), FOMO cohort: beijing (135), FOMO cohort: abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), FOMO cohort: ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), FOMO cohort: cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), fomo_wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), fomo_yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), fomo_nigerian (139), OASIS-2 (longitudinal) (138), fomo_hbnssi (137), fomo_beijing (135), fomo_abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), fomo_ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), fomo_cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F37" s="8" t="n">
@@ -9967,7 +10435,7 @@
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), FOMO cohort: wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), FOMO cohort: yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), FOMO cohort: nigerian (139), OASIS-2 (longitudinal) (138), FOMO cohort: hbnssi (137), FOMO cohort: beijing (135), FOMO cohort: abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), FOMO cohort: ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), FOMO cohort: cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), fomo_wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), fomo_yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), fomo_nigerian (139), OASIS-2 (longitudinal) (138), fomo_hbnssi (137), fomo_beijing (135), fomo_abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), fomo_ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), fomo_cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F38" s="8" t="n">
@@ -10001,7 +10469,7 @@
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), FOMO cohort: wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), FOMO cohort: yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), FOMO cohort: nigerian (139), OASIS-2 (longitudinal) (138), FOMO cohort: hbnssi (137), FOMO cohort: beijing (135), FOMO cohort: abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), FOMO cohort: ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), FOMO cohort: cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), Infant MRI (FOMO) (691), ABIDE I (640), AOMIC ID1000 (558), WAND (FOMO) (495), fomo_wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), fomo_yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), fomo_nigerian (139), OASIS-2 (longitudinal) (138), fomo_hbnssi (137), fomo_beijing (135), fomo_abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), fomo_ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), fomo_cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F39" s="8" t="n">
@@ -10035,7 +10503,7 @@
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (25,058), Healthy Brain Network (FOMO) (5,383), NKI-Rockland (FOMO) (3,426), CoRR (FOMO) (2,001), SLIM longitudinal (FOMO) (771), WAND (FOMO) (597), BrainLat (FOMO) (419), FOMO cohort: nigerian (203), Cuban Human Brain Mapping (FOMO) (153), FOMO cohort: hbnssi (137), FOMO cohort: beijing (135), FOMO cohort: wayne (134), ACPI (FOMO) (123), FOMO cohort: ageility (98), FOMO cohort: yale_highres (93), AHEAD 7T (FOMO) (79), FOMO cohort: cunmet (45), Tao Wu Parkinson's (FOMO) (30), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (25,058), Healthy Brain Network (FOMO) (5,383), NKI-Rockland (FOMO) (3,426), CoRR (FOMO) (2,001), SLIM longitudinal (FOMO) (771), WAND (FOMO) (597), BrainLat (FOMO) (419), fomo_nigerian (203), Cuban Human Brain Mapping (FOMO) (153), fomo_hbnssi (137), fomo_beijing (135), fomo_wayne (134), ACPI (FOMO) (123), fomo_ageility (98), fomo_yale_highres (93), AHEAD 7T (FOMO) (79), fomo_cunmet (45), Tao Wu Parkinson's (FOMO) (30), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F40" s="8" t="n">
@@ -10201,7 +10669,7 @@
       </c>
       <c r="E45" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F45" s="8" t="n">
@@ -10235,7 +10703,7 @@
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F46" s="8" t="n">
@@ -10269,7 +10737,7 @@
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F47" s="8" t="n">
@@ -10303,7 +10771,7 @@
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F48" s="8" t="n">
@@ -10337,7 +10805,7 @@
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F49" s="8" t="n">
@@ -10371,7 +10839,7 @@
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F50" s="8" t="n">
@@ -10405,7 +10873,7 @@
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F51" s="8" t="n">
@@ -10439,7 +10907,7 @@
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F52" s="8" t="n">
@@ -10473,7 +10941,7 @@
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F53" s="8" t="n">
@@ -10507,7 +10975,7 @@
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F54" s="8" t="n">
@@ -10541,7 +11009,7 @@
       </c>
       <c r="E55" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F55" s="8" t="n">
@@ -10575,7 +11043,7 @@
       </c>
       <c r="E56" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F56" s="8" t="n">
@@ -10609,7 +11077,7 @@
       </c>
       <c r="E57" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F57" s="8" t="n">
@@ -10643,7 +11111,7 @@
       </c>
       <c r="E58" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F58" s="8" t="n">
@@ -10677,7 +11145,7 @@
       </c>
       <c r="E59" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F59" s="8" t="n">
@@ -10711,7 +11179,7 @@
       </c>
       <c r="E60" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F60" s="8" t="n">
@@ -10745,7 +11213,7 @@
       </c>
       <c r="E61" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F61" s="8" t="n">
@@ -10779,7 +11247,7 @@
       </c>
       <c r="E62" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), FOMO cohort: wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), FOMO cohort: yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), FOMO cohort: beijing (107), FOMO cohort: nigerian (105), ACPI (FOMO) (98), FOMO cohort: ageility (98), FOMO cohort: abd (91), Pixar (OpenNeuro ds000228) (87), FOMO cohort: hbnssi (84), MICA-MICs (FOMO) (36), FOMO cohort: cunmet (35), Tao Wu Parkinson's (FOMO) (29), FOMO cohort: cleveland (23)</t>
+          <t>NKI-Rockland (FOMO) (2,991), Yale brain metastases (FOMO) (2,876), BraTS glioma (2021 / 2023 / 2024 GLI) (2,583), Healthy Brain Network (FOMO) (2,244), BraTS-MEN 2023 (2,026), CoRR (FOMO) (1,583), SLIM longitudinal (FOMO) (700), IXI (692), ABIDE I (630), AOMIC ID1000 (558), WAND (FOMO) (488), RSNA Intracranial Hemorrhage 2019 (448), fomo_wayne (422), BraTS-GoAT 2024 (403), BrainLat (FOMO) (350), Infant MRI (FOMO) (288), BraTS-PED 2023 (245), OASIS-1 (244), fomo_yale_highres (195), M4Raw low-field (FOMO) (194), OASIS-2 (longitudinal) (137), AOMIC PIOP2 (125), AOMIC PIOP1 (117), Cuban Human Brain Mapping (FOMO) (114), fomo_beijing (107), fomo_nigerian (105), ACPI (FOMO) (98), fomo_ageility (98), fomo_abd (91), Pixar (OpenNeuro ds000228) (87), fomo_hbnssi (84), MICA-MICs (FOMO) (36), fomo_cunmet (35), Tao Wu Parkinson's (FOMO) (29), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F62" s="8" t="n">
@@ -10813,7 +11281,7 @@
       </c>
       <c r="E63" s="7" t="inlineStr">
         <is>
-          <t>NKI-Rockland (FOMO) (2,529), Healthy Brain Network (FOMO) (2,113), IXI (433), M4Raw low-field (FOMO) (294), FOMO cohort: nigerian (104), BrainLat (FOMO) (31)</t>
+          <t>NKI-Rockland (FOMO) (2,529), Healthy Brain Network (FOMO) (2,113), IXI (433), M4Raw low-field (FOMO) (294), fomo_nigerian (104), BrainLat (FOMO) (31)</t>
         </is>
       </c>
       <c r="F63" s="8" t="n">
@@ -10915,7 +11383,7 @@
       </c>
       <c r="E66" s="7" t="inlineStr">
         <is>
-          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), ABIDE I (640), Infant MRI (FOMO) (627), AOMIC ID1000 (558), WAND (FOMO) (495), FOMO cohort: wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), FOMO cohort: yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), FOMO cohort: nigerian (139), OASIS-2 (longitudinal) (138), FOMO cohort: hbnssi (137), FOMO cohort: beijing (135), FOMO cohort: abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), FOMO cohort: ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), FOMO cohort: cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), FOMO cohort: cleveland (23)</t>
+          <t>Yale brain metastases (FOMO) (3,111), NKI-Rockland (FOMO) (3,074), BraTS glioma (2021 / 2023 / 2024 GLI) (2,736), Healthy Brain Network (FOMO) (2,575), BraTS-MEN 2023 (2,149), RSNA Intracranial Hemorrhage 2019 (1,708), CoRR (FOMO) (1,595), SLIM longitudinal (FOMO) (771), IXI (692), ABIDE I (640), Infant MRI (FOMO) (627), AOMIC ID1000 (558), WAND (FOMO) (495), fomo_wayne (449), BraTS-GoAT 2024 (419), BrainLat (FOMO) (358), M4Raw low-field (FOMO) (347), BraTS-PED 2023 (325), OASIS-1 (246), fomo_yale_highres (198), Cuban Human Brain Mapping (FOMO) (153), fomo_nigerian (139), OASIS-2 (longitudinal) (138), fomo_hbnssi (137), fomo_beijing (135), fomo_abd (131), AOMIC PIOP2 (125), AOMIC PIOP1 (117), ACPI (FOMO) (102), fomo_ageility (98), Pixar (OpenNeuro ds000228) (87), AHEAD 7T (FOMO) (79), fomo_cunmet (45), MICA-MICs (FOMO) (37), Tao Wu Parkinson's (FOMO) (30), fomo_cleveland (23)</t>
         </is>
       </c>
       <c r="F66" s="8" t="n">
@@ -11067,7 +11535,7 @@
       </c>
       <c r="E70" s="7" t="inlineStr">
         <is>
-          <t>ACPI (FOMO) (123), FOMO cohort: cunmet (45)</t>
+          <t>ACPI (FOMO) (123), fomo_cunmet (45)</t>
         </is>
       </c>
       <c r="F70" s="8" t="n">
@@ -11188,7 +11656,7 @@
         <v>562</v>
       </c>
       <c r="G73" s="8" t="n">
-        <v>198</v>
+        <v>150</v>
       </c>
       <c r="H73" s="7" t="inlineStr">
         <is>
@@ -11323,7 +11791,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -11350,7 +11818,7 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>2026-10-28 from the store index (volumes.csv, sha1 1ab77c50), labels/multitask_v2, brain.downstream.tasks and runs/bench/compare_v2.csv.</t>
+          <t>2026-10-29 from the store index (volumes.csv, sha1 59c96450), labels/multitask_v2, brain.downstream.tasks and runs/bench/compare_v2.csv.</t>
         </is>
       </c>
     </row>
@@ -11362,7 +11830,7 @@
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>In store: preprocessed and indexed. In pool, not prepared: raw archive downloaded. Access granted / Apply / Public download: not yet downloaded. Candidate: under consideration. Unidentified: named by a paper but not found.</t>
+          <t>In store: preprocessed and indexed. In store, not indexed: preprocessed, waiting for the next index rebuild. Prep running: preprocessing in progress. Deleted: downloaded earlier, removed. In pool, not prepared: raw archive downloaded. Access granted / Apply / Public download: not yet downloaded. Candidate: under consideration. Unidentified: named by a paper but not found.</t>
         </is>
       </c>
     </row>
@@ -11426,8 +11894,20 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>Label numbering</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Tumour masks are stored in BraTS 2023 numbering (1 necrosis / non-enhancing core, 2 oedema, 3 enhancing, 4 resection cavity in BraTS 2024); UCSF-PDGM / UPENN-GBM shipped 4 = enhancing and are remapped (pipeline.SEG_REMAP). Audit 2026-10-29: runs/diagnostics/tumor_label_semantics.py.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:B8"/>
+  <autoFilter ref="A1:B9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>